<commit_message>
align product with 365-day health tracker benchmark
</commit_message>
<xml_diff>
--- a/acha-outdoor-fat-loss-tracker-v1.xlsx
+++ b/acha-outdoor-fat-loss-tracker-v1.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="每週回顧" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'每日記錄'!$A$4:$N$204</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'每日記錄'!$A$4:$N$369</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -531,14 +531,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>阿茶外食減脂表｜Google Sheets 個人版</t>
+          <t>阿茶 365 天外食減脂表｜Google Sheets 個人版</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>不用備餐、不用先算很多卡路里，先把今天這一餐記下來。</t>
+          <t>365 天記錄外食、體重、腰圍與習慣，不用一次做到完美。</t>
         </is>
       </c>
     </row>
@@ -572,7 +572,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>到「每日記錄」輸入今天吃的餐點與情境</t>
+          <t>到「每日記錄」輸入今天的餐點、體重與習慣</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -582,7 +582,7 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>先記一餐就好</t>
+          <t>365 天慢慢累積</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>每週到「每週回顧」看完成天數與記錄餐數</t>
+          <t>每週到「每週回顧」看見記錄與身體變化</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -743,7 +743,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N204"/>
+  <dimension ref="A1:N369"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -5248,8 +5248,3638 @@
         <v/>
       </c>
     </row>
+    <row r="205">
+      <c r="A205" s="10" t="n"/>
+      <c r="B205" s="11" t="n"/>
+      <c r="C205" s="11" t="n"/>
+      <c r="D205" s="11" t="n"/>
+      <c r="E205" s="11" t="n"/>
+      <c r="F205" s="11" t="n"/>
+      <c r="G205" s="11" t="n"/>
+      <c r="H205" s="11" t="n"/>
+      <c r="I205" s="11" t="n"/>
+      <c r="J205" s="12" t="n"/>
+      <c r="K205" s="12" t="n"/>
+      <c r="L205" s="13">
+        <f>COUNTIF(E205:G205,"有")+IF(H205&gt;=6,1,0)+IF(I205&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M205" s="11" t="n"/>
+      <c r="N205" s="13">
+        <f>IF(COUNTA(A205:G205)=0,"",IF(L205&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="10" t="n"/>
+      <c r="B206" s="11" t="n"/>
+      <c r="C206" s="11" t="n"/>
+      <c r="D206" s="11" t="n"/>
+      <c r="E206" s="11" t="n"/>
+      <c r="F206" s="11" t="n"/>
+      <c r="G206" s="11" t="n"/>
+      <c r="H206" s="11" t="n"/>
+      <c r="I206" s="11" t="n"/>
+      <c r="J206" s="12" t="n"/>
+      <c r="K206" s="12" t="n"/>
+      <c r="L206" s="13">
+        <f>COUNTIF(E206:G206,"有")+IF(H206&gt;=6,1,0)+IF(I206&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M206" s="11" t="n"/>
+      <c r="N206" s="13">
+        <f>IF(COUNTA(A206:G206)=0,"",IF(L206&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="10" t="n"/>
+      <c r="B207" s="11" t="n"/>
+      <c r="C207" s="11" t="n"/>
+      <c r="D207" s="11" t="n"/>
+      <c r="E207" s="11" t="n"/>
+      <c r="F207" s="11" t="n"/>
+      <c r="G207" s="11" t="n"/>
+      <c r="H207" s="11" t="n"/>
+      <c r="I207" s="11" t="n"/>
+      <c r="J207" s="12" t="n"/>
+      <c r="K207" s="12" t="n"/>
+      <c r="L207" s="13">
+        <f>COUNTIF(E207:G207,"有")+IF(H207&gt;=6,1,0)+IF(I207&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M207" s="11" t="n"/>
+      <c r="N207" s="13">
+        <f>IF(COUNTA(A207:G207)=0,"",IF(L207&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="10" t="n"/>
+      <c r="B208" s="11" t="n"/>
+      <c r="C208" s="11" t="n"/>
+      <c r="D208" s="11" t="n"/>
+      <c r="E208" s="11" t="n"/>
+      <c r="F208" s="11" t="n"/>
+      <c r="G208" s="11" t="n"/>
+      <c r="H208" s="11" t="n"/>
+      <c r="I208" s="11" t="n"/>
+      <c r="J208" s="12" t="n"/>
+      <c r="K208" s="12" t="n"/>
+      <c r="L208" s="13">
+        <f>COUNTIF(E208:G208,"有")+IF(H208&gt;=6,1,0)+IF(I208&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M208" s="11" t="n"/>
+      <c r="N208" s="13">
+        <f>IF(COUNTA(A208:G208)=0,"",IF(L208&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="10" t="n"/>
+      <c r="B209" s="11" t="n"/>
+      <c r="C209" s="11" t="n"/>
+      <c r="D209" s="11" t="n"/>
+      <c r="E209" s="11" t="n"/>
+      <c r="F209" s="11" t="n"/>
+      <c r="G209" s="11" t="n"/>
+      <c r="H209" s="11" t="n"/>
+      <c r="I209" s="11" t="n"/>
+      <c r="J209" s="12" t="n"/>
+      <c r="K209" s="12" t="n"/>
+      <c r="L209" s="13">
+        <f>COUNTIF(E209:G209,"有")+IF(H209&gt;=6,1,0)+IF(I209&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M209" s="11" t="n"/>
+      <c r="N209" s="13">
+        <f>IF(COUNTA(A209:G209)=0,"",IF(L209&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="10" t="n"/>
+      <c r="B210" s="11" t="n"/>
+      <c r="C210" s="11" t="n"/>
+      <c r="D210" s="11" t="n"/>
+      <c r="E210" s="11" t="n"/>
+      <c r="F210" s="11" t="n"/>
+      <c r="G210" s="11" t="n"/>
+      <c r="H210" s="11" t="n"/>
+      <c r="I210" s="11" t="n"/>
+      <c r="J210" s="12" t="n"/>
+      <c r="K210" s="12" t="n"/>
+      <c r="L210" s="13">
+        <f>COUNTIF(E210:G210,"有")+IF(H210&gt;=6,1,0)+IF(I210&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M210" s="11" t="n"/>
+      <c r="N210" s="13">
+        <f>IF(COUNTA(A210:G210)=0,"",IF(L210&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="10" t="n"/>
+      <c r="B211" s="11" t="n"/>
+      <c r="C211" s="11" t="n"/>
+      <c r="D211" s="11" t="n"/>
+      <c r="E211" s="11" t="n"/>
+      <c r="F211" s="11" t="n"/>
+      <c r="G211" s="11" t="n"/>
+      <c r="H211" s="11" t="n"/>
+      <c r="I211" s="11" t="n"/>
+      <c r="J211" s="12" t="n"/>
+      <c r="K211" s="12" t="n"/>
+      <c r="L211" s="13">
+        <f>COUNTIF(E211:G211,"有")+IF(H211&gt;=6,1,0)+IF(I211&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M211" s="11" t="n"/>
+      <c r="N211" s="13">
+        <f>IF(COUNTA(A211:G211)=0,"",IF(L211&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="10" t="n"/>
+      <c r="B212" s="11" t="n"/>
+      <c r="C212" s="11" t="n"/>
+      <c r="D212" s="11" t="n"/>
+      <c r="E212" s="11" t="n"/>
+      <c r="F212" s="11" t="n"/>
+      <c r="G212" s="11" t="n"/>
+      <c r="H212" s="11" t="n"/>
+      <c r="I212" s="11" t="n"/>
+      <c r="J212" s="12" t="n"/>
+      <c r="K212" s="12" t="n"/>
+      <c r="L212" s="13">
+        <f>COUNTIF(E212:G212,"有")+IF(H212&gt;=6,1,0)+IF(I212&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M212" s="11" t="n"/>
+      <c r="N212" s="13">
+        <f>IF(COUNTA(A212:G212)=0,"",IF(L212&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="10" t="n"/>
+      <c r="B213" s="11" t="n"/>
+      <c r="C213" s="11" t="n"/>
+      <c r="D213" s="11" t="n"/>
+      <c r="E213" s="11" t="n"/>
+      <c r="F213" s="11" t="n"/>
+      <c r="G213" s="11" t="n"/>
+      <c r="H213" s="11" t="n"/>
+      <c r="I213" s="11" t="n"/>
+      <c r="J213" s="12" t="n"/>
+      <c r="K213" s="12" t="n"/>
+      <c r="L213" s="13">
+        <f>COUNTIF(E213:G213,"有")+IF(H213&gt;=6,1,0)+IF(I213&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M213" s="11" t="n"/>
+      <c r="N213" s="13">
+        <f>IF(COUNTA(A213:G213)=0,"",IF(L213&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="10" t="n"/>
+      <c r="B214" s="11" t="n"/>
+      <c r="C214" s="11" t="n"/>
+      <c r="D214" s="11" t="n"/>
+      <c r="E214" s="11" t="n"/>
+      <c r="F214" s="11" t="n"/>
+      <c r="G214" s="11" t="n"/>
+      <c r="H214" s="11" t="n"/>
+      <c r="I214" s="11" t="n"/>
+      <c r="J214" s="12" t="n"/>
+      <c r="K214" s="12" t="n"/>
+      <c r="L214" s="13">
+        <f>COUNTIF(E214:G214,"有")+IF(H214&gt;=6,1,0)+IF(I214&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M214" s="11" t="n"/>
+      <c r="N214" s="13">
+        <f>IF(COUNTA(A214:G214)=0,"",IF(L214&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="10" t="n"/>
+      <c r="B215" s="11" t="n"/>
+      <c r="C215" s="11" t="n"/>
+      <c r="D215" s="11" t="n"/>
+      <c r="E215" s="11" t="n"/>
+      <c r="F215" s="11" t="n"/>
+      <c r="G215" s="11" t="n"/>
+      <c r="H215" s="11" t="n"/>
+      <c r="I215" s="11" t="n"/>
+      <c r="J215" s="12" t="n"/>
+      <c r="K215" s="12" t="n"/>
+      <c r="L215" s="13">
+        <f>COUNTIF(E215:G215,"有")+IF(H215&gt;=6,1,0)+IF(I215&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M215" s="11" t="n"/>
+      <c r="N215" s="13">
+        <f>IF(COUNTA(A215:G215)=0,"",IF(L215&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="10" t="n"/>
+      <c r="B216" s="11" t="n"/>
+      <c r="C216" s="11" t="n"/>
+      <c r="D216" s="11" t="n"/>
+      <c r="E216" s="11" t="n"/>
+      <c r="F216" s="11" t="n"/>
+      <c r="G216" s="11" t="n"/>
+      <c r="H216" s="11" t="n"/>
+      <c r="I216" s="11" t="n"/>
+      <c r="J216" s="12" t="n"/>
+      <c r="K216" s="12" t="n"/>
+      <c r="L216" s="13">
+        <f>COUNTIF(E216:G216,"有")+IF(H216&gt;=6,1,0)+IF(I216&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M216" s="11" t="n"/>
+      <c r="N216" s="13">
+        <f>IF(COUNTA(A216:G216)=0,"",IF(L216&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="10" t="n"/>
+      <c r="B217" s="11" t="n"/>
+      <c r="C217" s="11" t="n"/>
+      <c r="D217" s="11" t="n"/>
+      <c r="E217" s="11" t="n"/>
+      <c r="F217" s="11" t="n"/>
+      <c r="G217" s="11" t="n"/>
+      <c r="H217" s="11" t="n"/>
+      <c r="I217" s="11" t="n"/>
+      <c r="J217" s="12" t="n"/>
+      <c r="K217" s="12" t="n"/>
+      <c r="L217" s="13">
+        <f>COUNTIF(E217:G217,"有")+IF(H217&gt;=6,1,0)+IF(I217&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M217" s="11" t="n"/>
+      <c r="N217" s="13">
+        <f>IF(COUNTA(A217:G217)=0,"",IF(L217&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="10" t="n"/>
+      <c r="B218" s="11" t="n"/>
+      <c r="C218" s="11" t="n"/>
+      <c r="D218" s="11" t="n"/>
+      <c r="E218" s="11" t="n"/>
+      <c r="F218" s="11" t="n"/>
+      <c r="G218" s="11" t="n"/>
+      <c r="H218" s="11" t="n"/>
+      <c r="I218" s="11" t="n"/>
+      <c r="J218" s="12" t="n"/>
+      <c r="K218" s="12" t="n"/>
+      <c r="L218" s="13">
+        <f>COUNTIF(E218:G218,"有")+IF(H218&gt;=6,1,0)+IF(I218&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M218" s="11" t="n"/>
+      <c r="N218" s="13">
+        <f>IF(COUNTA(A218:G218)=0,"",IF(L218&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="10" t="n"/>
+      <c r="B219" s="11" t="n"/>
+      <c r="C219" s="11" t="n"/>
+      <c r="D219" s="11" t="n"/>
+      <c r="E219" s="11" t="n"/>
+      <c r="F219" s="11" t="n"/>
+      <c r="G219" s="11" t="n"/>
+      <c r="H219" s="11" t="n"/>
+      <c r="I219" s="11" t="n"/>
+      <c r="J219" s="12" t="n"/>
+      <c r="K219" s="12" t="n"/>
+      <c r="L219" s="13">
+        <f>COUNTIF(E219:G219,"有")+IF(H219&gt;=6,1,0)+IF(I219&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M219" s="11" t="n"/>
+      <c r="N219" s="13">
+        <f>IF(COUNTA(A219:G219)=0,"",IF(L219&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="10" t="n"/>
+      <c r="B220" s="11" t="n"/>
+      <c r="C220" s="11" t="n"/>
+      <c r="D220" s="11" t="n"/>
+      <c r="E220" s="11" t="n"/>
+      <c r="F220" s="11" t="n"/>
+      <c r="G220" s="11" t="n"/>
+      <c r="H220" s="11" t="n"/>
+      <c r="I220" s="11" t="n"/>
+      <c r="J220" s="12" t="n"/>
+      <c r="K220" s="12" t="n"/>
+      <c r="L220" s="13">
+        <f>COUNTIF(E220:G220,"有")+IF(H220&gt;=6,1,0)+IF(I220&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M220" s="11" t="n"/>
+      <c r="N220" s="13">
+        <f>IF(COUNTA(A220:G220)=0,"",IF(L220&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="10" t="n"/>
+      <c r="B221" s="11" t="n"/>
+      <c r="C221" s="11" t="n"/>
+      <c r="D221" s="11" t="n"/>
+      <c r="E221" s="11" t="n"/>
+      <c r="F221" s="11" t="n"/>
+      <c r="G221" s="11" t="n"/>
+      <c r="H221" s="11" t="n"/>
+      <c r="I221" s="11" t="n"/>
+      <c r="J221" s="12" t="n"/>
+      <c r="K221" s="12" t="n"/>
+      <c r="L221" s="13">
+        <f>COUNTIF(E221:G221,"有")+IF(H221&gt;=6,1,0)+IF(I221&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M221" s="11" t="n"/>
+      <c r="N221" s="13">
+        <f>IF(COUNTA(A221:G221)=0,"",IF(L221&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="10" t="n"/>
+      <c r="B222" s="11" t="n"/>
+      <c r="C222" s="11" t="n"/>
+      <c r="D222" s="11" t="n"/>
+      <c r="E222" s="11" t="n"/>
+      <c r="F222" s="11" t="n"/>
+      <c r="G222" s="11" t="n"/>
+      <c r="H222" s="11" t="n"/>
+      <c r="I222" s="11" t="n"/>
+      <c r="J222" s="12" t="n"/>
+      <c r="K222" s="12" t="n"/>
+      <c r="L222" s="13">
+        <f>COUNTIF(E222:G222,"有")+IF(H222&gt;=6,1,0)+IF(I222&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M222" s="11" t="n"/>
+      <c r="N222" s="13">
+        <f>IF(COUNTA(A222:G222)=0,"",IF(L222&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="10" t="n"/>
+      <c r="B223" s="11" t="n"/>
+      <c r="C223" s="11" t="n"/>
+      <c r="D223" s="11" t="n"/>
+      <c r="E223" s="11" t="n"/>
+      <c r="F223" s="11" t="n"/>
+      <c r="G223" s="11" t="n"/>
+      <c r="H223" s="11" t="n"/>
+      <c r="I223" s="11" t="n"/>
+      <c r="J223" s="12" t="n"/>
+      <c r="K223" s="12" t="n"/>
+      <c r="L223" s="13">
+        <f>COUNTIF(E223:G223,"有")+IF(H223&gt;=6,1,0)+IF(I223&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M223" s="11" t="n"/>
+      <c r="N223" s="13">
+        <f>IF(COUNTA(A223:G223)=0,"",IF(L223&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="10" t="n"/>
+      <c r="B224" s="11" t="n"/>
+      <c r="C224" s="11" t="n"/>
+      <c r="D224" s="11" t="n"/>
+      <c r="E224" s="11" t="n"/>
+      <c r="F224" s="11" t="n"/>
+      <c r="G224" s="11" t="n"/>
+      <c r="H224" s="11" t="n"/>
+      <c r="I224" s="11" t="n"/>
+      <c r="J224" s="12" t="n"/>
+      <c r="K224" s="12" t="n"/>
+      <c r="L224" s="13">
+        <f>COUNTIF(E224:G224,"有")+IF(H224&gt;=6,1,0)+IF(I224&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M224" s="11" t="n"/>
+      <c r="N224" s="13">
+        <f>IF(COUNTA(A224:G224)=0,"",IF(L224&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="10" t="n"/>
+      <c r="B225" s="11" t="n"/>
+      <c r="C225" s="11" t="n"/>
+      <c r="D225" s="11" t="n"/>
+      <c r="E225" s="11" t="n"/>
+      <c r="F225" s="11" t="n"/>
+      <c r="G225" s="11" t="n"/>
+      <c r="H225" s="11" t="n"/>
+      <c r="I225" s="11" t="n"/>
+      <c r="J225" s="12" t="n"/>
+      <c r="K225" s="12" t="n"/>
+      <c r="L225" s="13">
+        <f>COUNTIF(E225:G225,"有")+IF(H225&gt;=6,1,0)+IF(I225&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M225" s="11" t="n"/>
+      <c r="N225" s="13">
+        <f>IF(COUNTA(A225:G225)=0,"",IF(L225&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="10" t="n"/>
+      <c r="B226" s="11" t="n"/>
+      <c r="C226" s="11" t="n"/>
+      <c r="D226" s="11" t="n"/>
+      <c r="E226" s="11" t="n"/>
+      <c r="F226" s="11" t="n"/>
+      <c r="G226" s="11" t="n"/>
+      <c r="H226" s="11" t="n"/>
+      <c r="I226" s="11" t="n"/>
+      <c r="J226" s="12" t="n"/>
+      <c r="K226" s="12" t="n"/>
+      <c r="L226" s="13">
+        <f>COUNTIF(E226:G226,"有")+IF(H226&gt;=6,1,0)+IF(I226&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M226" s="11" t="n"/>
+      <c r="N226" s="13">
+        <f>IF(COUNTA(A226:G226)=0,"",IF(L226&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="10" t="n"/>
+      <c r="B227" s="11" t="n"/>
+      <c r="C227" s="11" t="n"/>
+      <c r="D227" s="11" t="n"/>
+      <c r="E227" s="11" t="n"/>
+      <c r="F227" s="11" t="n"/>
+      <c r="G227" s="11" t="n"/>
+      <c r="H227" s="11" t="n"/>
+      <c r="I227" s="11" t="n"/>
+      <c r="J227" s="12" t="n"/>
+      <c r="K227" s="12" t="n"/>
+      <c r="L227" s="13">
+        <f>COUNTIF(E227:G227,"有")+IF(H227&gt;=6,1,0)+IF(I227&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M227" s="11" t="n"/>
+      <c r="N227" s="13">
+        <f>IF(COUNTA(A227:G227)=0,"",IF(L227&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="10" t="n"/>
+      <c r="B228" s="11" t="n"/>
+      <c r="C228" s="11" t="n"/>
+      <c r="D228" s="11" t="n"/>
+      <c r="E228" s="11" t="n"/>
+      <c r="F228" s="11" t="n"/>
+      <c r="G228" s="11" t="n"/>
+      <c r="H228" s="11" t="n"/>
+      <c r="I228" s="11" t="n"/>
+      <c r="J228" s="12" t="n"/>
+      <c r="K228" s="12" t="n"/>
+      <c r="L228" s="13">
+        <f>COUNTIF(E228:G228,"有")+IF(H228&gt;=6,1,0)+IF(I228&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M228" s="11" t="n"/>
+      <c r="N228" s="13">
+        <f>IF(COUNTA(A228:G228)=0,"",IF(L228&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="10" t="n"/>
+      <c r="B229" s="11" t="n"/>
+      <c r="C229" s="11" t="n"/>
+      <c r="D229" s="11" t="n"/>
+      <c r="E229" s="11" t="n"/>
+      <c r="F229" s="11" t="n"/>
+      <c r="G229" s="11" t="n"/>
+      <c r="H229" s="11" t="n"/>
+      <c r="I229" s="11" t="n"/>
+      <c r="J229" s="12" t="n"/>
+      <c r="K229" s="12" t="n"/>
+      <c r="L229" s="13">
+        <f>COUNTIF(E229:G229,"有")+IF(H229&gt;=6,1,0)+IF(I229&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M229" s="11" t="n"/>
+      <c r="N229" s="13">
+        <f>IF(COUNTA(A229:G229)=0,"",IF(L229&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="10" t="n"/>
+      <c r="B230" s="11" t="n"/>
+      <c r="C230" s="11" t="n"/>
+      <c r="D230" s="11" t="n"/>
+      <c r="E230" s="11" t="n"/>
+      <c r="F230" s="11" t="n"/>
+      <c r="G230" s="11" t="n"/>
+      <c r="H230" s="11" t="n"/>
+      <c r="I230" s="11" t="n"/>
+      <c r="J230" s="12" t="n"/>
+      <c r="K230" s="12" t="n"/>
+      <c r="L230" s="13">
+        <f>COUNTIF(E230:G230,"有")+IF(H230&gt;=6,1,0)+IF(I230&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M230" s="11" t="n"/>
+      <c r="N230" s="13">
+        <f>IF(COUNTA(A230:G230)=0,"",IF(L230&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" s="10" t="n"/>
+      <c r="B231" s="11" t="n"/>
+      <c r="C231" s="11" t="n"/>
+      <c r="D231" s="11" t="n"/>
+      <c r="E231" s="11" t="n"/>
+      <c r="F231" s="11" t="n"/>
+      <c r="G231" s="11" t="n"/>
+      <c r="H231" s="11" t="n"/>
+      <c r="I231" s="11" t="n"/>
+      <c r="J231" s="12" t="n"/>
+      <c r="K231" s="12" t="n"/>
+      <c r="L231" s="13">
+        <f>COUNTIF(E231:G231,"有")+IF(H231&gt;=6,1,0)+IF(I231&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M231" s="11" t="n"/>
+      <c r="N231" s="13">
+        <f>IF(COUNTA(A231:G231)=0,"",IF(L231&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="10" t="n"/>
+      <c r="B232" s="11" t="n"/>
+      <c r="C232" s="11" t="n"/>
+      <c r="D232" s="11" t="n"/>
+      <c r="E232" s="11" t="n"/>
+      <c r="F232" s="11" t="n"/>
+      <c r="G232" s="11" t="n"/>
+      <c r="H232" s="11" t="n"/>
+      <c r="I232" s="11" t="n"/>
+      <c r="J232" s="12" t="n"/>
+      <c r="K232" s="12" t="n"/>
+      <c r="L232" s="13">
+        <f>COUNTIF(E232:G232,"有")+IF(H232&gt;=6,1,0)+IF(I232&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M232" s="11" t="n"/>
+      <c r="N232" s="13">
+        <f>IF(COUNTA(A232:G232)=0,"",IF(L232&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="10" t="n"/>
+      <c r="B233" s="11" t="n"/>
+      <c r="C233" s="11" t="n"/>
+      <c r="D233" s="11" t="n"/>
+      <c r="E233" s="11" t="n"/>
+      <c r="F233" s="11" t="n"/>
+      <c r="G233" s="11" t="n"/>
+      <c r="H233" s="11" t="n"/>
+      <c r="I233" s="11" t="n"/>
+      <c r="J233" s="12" t="n"/>
+      <c r="K233" s="12" t="n"/>
+      <c r="L233" s="13">
+        <f>COUNTIF(E233:G233,"有")+IF(H233&gt;=6,1,0)+IF(I233&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M233" s="11" t="n"/>
+      <c r="N233" s="13">
+        <f>IF(COUNTA(A233:G233)=0,"",IF(L233&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="10" t="n"/>
+      <c r="B234" s="11" t="n"/>
+      <c r="C234" s="11" t="n"/>
+      <c r="D234" s="11" t="n"/>
+      <c r="E234" s="11" t="n"/>
+      <c r="F234" s="11" t="n"/>
+      <c r="G234" s="11" t="n"/>
+      <c r="H234" s="11" t="n"/>
+      <c r="I234" s="11" t="n"/>
+      <c r="J234" s="12" t="n"/>
+      <c r="K234" s="12" t="n"/>
+      <c r="L234" s="13">
+        <f>COUNTIF(E234:G234,"有")+IF(H234&gt;=6,1,0)+IF(I234&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M234" s="11" t="n"/>
+      <c r="N234" s="13">
+        <f>IF(COUNTA(A234:G234)=0,"",IF(L234&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" s="10" t="n"/>
+      <c r="B235" s="11" t="n"/>
+      <c r="C235" s="11" t="n"/>
+      <c r="D235" s="11" t="n"/>
+      <c r="E235" s="11" t="n"/>
+      <c r="F235" s="11" t="n"/>
+      <c r="G235" s="11" t="n"/>
+      <c r="H235" s="11" t="n"/>
+      <c r="I235" s="11" t="n"/>
+      <c r="J235" s="12" t="n"/>
+      <c r="K235" s="12" t="n"/>
+      <c r="L235" s="13">
+        <f>COUNTIF(E235:G235,"有")+IF(H235&gt;=6,1,0)+IF(I235&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M235" s="11" t="n"/>
+      <c r="N235" s="13">
+        <f>IF(COUNTA(A235:G235)=0,"",IF(L235&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="10" t="n"/>
+      <c r="B236" s="11" t="n"/>
+      <c r="C236" s="11" t="n"/>
+      <c r="D236" s="11" t="n"/>
+      <c r="E236" s="11" t="n"/>
+      <c r="F236" s="11" t="n"/>
+      <c r="G236" s="11" t="n"/>
+      <c r="H236" s="11" t="n"/>
+      <c r="I236" s="11" t="n"/>
+      <c r="J236" s="12" t="n"/>
+      <c r="K236" s="12" t="n"/>
+      <c r="L236" s="13">
+        <f>COUNTIF(E236:G236,"有")+IF(H236&gt;=6,1,0)+IF(I236&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M236" s="11" t="n"/>
+      <c r="N236" s="13">
+        <f>IF(COUNTA(A236:G236)=0,"",IF(L236&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="10" t="n"/>
+      <c r="B237" s="11" t="n"/>
+      <c r="C237" s="11" t="n"/>
+      <c r="D237" s="11" t="n"/>
+      <c r="E237" s="11" t="n"/>
+      <c r="F237" s="11" t="n"/>
+      <c r="G237" s="11" t="n"/>
+      <c r="H237" s="11" t="n"/>
+      <c r="I237" s="11" t="n"/>
+      <c r="J237" s="12" t="n"/>
+      <c r="K237" s="12" t="n"/>
+      <c r="L237" s="13">
+        <f>COUNTIF(E237:G237,"有")+IF(H237&gt;=6,1,0)+IF(I237&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M237" s="11" t="n"/>
+      <c r="N237" s="13">
+        <f>IF(COUNTA(A237:G237)=0,"",IF(L237&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" s="10" t="n"/>
+      <c r="B238" s="11" t="n"/>
+      <c r="C238" s="11" t="n"/>
+      <c r="D238" s="11" t="n"/>
+      <c r="E238" s="11" t="n"/>
+      <c r="F238" s="11" t="n"/>
+      <c r="G238" s="11" t="n"/>
+      <c r="H238" s="11" t="n"/>
+      <c r="I238" s="11" t="n"/>
+      <c r="J238" s="12" t="n"/>
+      <c r="K238" s="12" t="n"/>
+      <c r="L238" s="13">
+        <f>COUNTIF(E238:G238,"有")+IF(H238&gt;=6,1,0)+IF(I238&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M238" s="11" t="n"/>
+      <c r="N238" s="13">
+        <f>IF(COUNTA(A238:G238)=0,"",IF(L238&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" s="10" t="n"/>
+      <c r="B239" s="11" t="n"/>
+      <c r="C239" s="11" t="n"/>
+      <c r="D239" s="11" t="n"/>
+      <c r="E239" s="11" t="n"/>
+      <c r="F239" s="11" t="n"/>
+      <c r="G239" s="11" t="n"/>
+      <c r="H239" s="11" t="n"/>
+      <c r="I239" s="11" t="n"/>
+      <c r="J239" s="12" t="n"/>
+      <c r="K239" s="12" t="n"/>
+      <c r="L239" s="13">
+        <f>COUNTIF(E239:G239,"有")+IF(H239&gt;=6,1,0)+IF(I239&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M239" s="11" t="n"/>
+      <c r="N239" s="13">
+        <f>IF(COUNTA(A239:G239)=0,"",IF(L239&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" s="10" t="n"/>
+      <c r="B240" s="11" t="n"/>
+      <c r="C240" s="11" t="n"/>
+      <c r="D240" s="11" t="n"/>
+      <c r="E240" s="11" t="n"/>
+      <c r="F240" s="11" t="n"/>
+      <c r="G240" s="11" t="n"/>
+      <c r="H240" s="11" t="n"/>
+      <c r="I240" s="11" t="n"/>
+      <c r="J240" s="12" t="n"/>
+      <c r="K240" s="12" t="n"/>
+      <c r="L240" s="13">
+        <f>COUNTIF(E240:G240,"有")+IF(H240&gt;=6,1,0)+IF(I240&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M240" s="11" t="n"/>
+      <c r="N240" s="13">
+        <f>IF(COUNTA(A240:G240)=0,"",IF(L240&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" s="10" t="n"/>
+      <c r="B241" s="11" t="n"/>
+      <c r="C241" s="11" t="n"/>
+      <c r="D241" s="11" t="n"/>
+      <c r="E241" s="11" t="n"/>
+      <c r="F241" s="11" t="n"/>
+      <c r="G241" s="11" t="n"/>
+      <c r="H241" s="11" t="n"/>
+      <c r="I241" s="11" t="n"/>
+      <c r="J241" s="12" t="n"/>
+      <c r="K241" s="12" t="n"/>
+      <c r="L241" s="13">
+        <f>COUNTIF(E241:G241,"有")+IF(H241&gt;=6,1,0)+IF(I241&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M241" s="11" t="n"/>
+      <c r="N241" s="13">
+        <f>IF(COUNTA(A241:G241)=0,"",IF(L241&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" s="10" t="n"/>
+      <c r="B242" s="11" t="n"/>
+      <c r="C242" s="11" t="n"/>
+      <c r="D242" s="11" t="n"/>
+      <c r="E242" s="11" t="n"/>
+      <c r="F242" s="11" t="n"/>
+      <c r="G242" s="11" t="n"/>
+      <c r="H242" s="11" t="n"/>
+      <c r="I242" s="11" t="n"/>
+      <c r="J242" s="12" t="n"/>
+      <c r="K242" s="12" t="n"/>
+      <c r="L242" s="13">
+        <f>COUNTIF(E242:G242,"有")+IF(H242&gt;=6,1,0)+IF(I242&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M242" s="11" t="n"/>
+      <c r="N242" s="13">
+        <f>IF(COUNTA(A242:G242)=0,"",IF(L242&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" s="10" t="n"/>
+      <c r="B243" s="11" t="n"/>
+      <c r="C243" s="11" t="n"/>
+      <c r="D243" s="11" t="n"/>
+      <c r="E243" s="11" t="n"/>
+      <c r="F243" s="11" t="n"/>
+      <c r="G243" s="11" t="n"/>
+      <c r="H243" s="11" t="n"/>
+      <c r="I243" s="11" t="n"/>
+      <c r="J243" s="12" t="n"/>
+      <c r="K243" s="12" t="n"/>
+      <c r="L243" s="13">
+        <f>COUNTIF(E243:G243,"有")+IF(H243&gt;=6,1,0)+IF(I243&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M243" s="11" t="n"/>
+      <c r="N243" s="13">
+        <f>IF(COUNTA(A243:G243)=0,"",IF(L243&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" s="10" t="n"/>
+      <c r="B244" s="11" t="n"/>
+      <c r="C244" s="11" t="n"/>
+      <c r="D244" s="11" t="n"/>
+      <c r="E244" s="11" t="n"/>
+      <c r="F244" s="11" t="n"/>
+      <c r="G244" s="11" t="n"/>
+      <c r="H244" s="11" t="n"/>
+      <c r="I244" s="11" t="n"/>
+      <c r="J244" s="12" t="n"/>
+      <c r="K244" s="12" t="n"/>
+      <c r="L244" s="13">
+        <f>COUNTIF(E244:G244,"有")+IF(H244&gt;=6,1,0)+IF(I244&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M244" s="11" t="n"/>
+      <c r="N244" s="13">
+        <f>IF(COUNTA(A244:G244)=0,"",IF(L244&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" s="10" t="n"/>
+      <c r="B245" s="11" t="n"/>
+      <c r="C245" s="11" t="n"/>
+      <c r="D245" s="11" t="n"/>
+      <c r="E245" s="11" t="n"/>
+      <c r="F245" s="11" t="n"/>
+      <c r="G245" s="11" t="n"/>
+      <c r="H245" s="11" t="n"/>
+      <c r="I245" s="11" t="n"/>
+      <c r="J245" s="12" t="n"/>
+      <c r="K245" s="12" t="n"/>
+      <c r="L245" s="13">
+        <f>COUNTIF(E245:G245,"有")+IF(H245&gt;=6,1,0)+IF(I245&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M245" s="11" t="n"/>
+      <c r="N245" s="13">
+        <f>IF(COUNTA(A245:G245)=0,"",IF(L245&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" s="10" t="n"/>
+      <c r="B246" s="11" t="n"/>
+      <c r="C246" s="11" t="n"/>
+      <c r="D246" s="11" t="n"/>
+      <c r="E246" s="11" t="n"/>
+      <c r="F246" s="11" t="n"/>
+      <c r="G246" s="11" t="n"/>
+      <c r="H246" s="11" t="n"/>
+      <c r="I246" s="11" t="n"/>
+      <c r="J246" s="12" t="n"/>
+      <c r="K246" s="12" t="n"/>
+      <c r="L246" s="13">
+        <f>COUNTIF(E246:G246,"有")+IF(H246&gt;=6,1,0)+IF(I246&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M246" s="11" t="n"/>
+      <c r="N246" s="13">
+        <f>IF(COUNTA(A246:G246)=0,"",IF(L246&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" s="10" t="n"/>
+      <c r="B247" s="11" t="n"/>
+      <c r="C247" s="11" t="n"/>
+      <c r="D247" s="11" t="n"/>
+      <c r="E247" s="11" t="n"/>
+      <c r="F247" s="11" t="n"/>
+      <c r="G247" s="11" t="n"/>
+      <c r="H247" s="11" t="n"/>
+      <c r="I247" s="11" t="n"/>
+      <c r="J247" s="12" t="n"/>
+      <c r="K247" s="12" t="n"/>
+      <c r="L247" s="13">
+        <f>COUNTIF(E247:G247,"有")+IF(H247&gt;=6,1,0)+IF(I247&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M247" s="11" t="n"/>
+      <c r="N247" s="13">
+        <f>IF(COUNTA(A247:G247)=0,"",IF(L247&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" s="10" t="n"/>
+      <c r="B248" s="11" t="n"/>
+      <c r="C248" s="11" t="n"/>
+      <c r="D248" s="11" t="n"/>
+      <c r="E248" s="11" t="n"/>
+      <c r="F248" s="11" t="n"/>
+      <c r="G248" s="11" t="n"/>
+      <c r="H248" s="11" t="n"/>
+      <c r="I248" s="11" t="n"/>
+      <c r="J248" s="12" t="n"/>
+      <c r="K248" s="12" t="n"/>
+      <c r="L248" s="13">
+        <f>COUNTIF(E248:G248,"有")+IF(H248&gt;=6,1,0)+IF(I248&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M248" s="11" t="n"/>
+      <c r="N248" s="13">
+        <f>IF(COUNTA(A248:G248)=0,"",IF(L248&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" s="10" t="n"/>
+      <c r="B249" s="11" t="n"/>
+      <c r="C249" s="11" t="n"/>
+      <c r="D249" s="11" t="n"/>
+      <c r="E249" s="11" t="n"/>
+      <c r="F249" s="11" t="n"/>
+      <c r="G249" s="11" t="n"/>
+      <c r="H249" s="11" t="n"/>
+      <c r="I249" s="11" t="n"/>
+      <c r="J249" s="12" t="n"/>
+      <c r="K249" s="12" t="n"/>
+      <c r="L249" s="13">
+        <f>COUNTIF(E249:G249,"有")+IF(H249&gt;=6,1,0)+IF(I249&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M249" s="11" t="n"/>
+      <c r="N249" s="13">
+        <f>IF(COUNTA(A249:G249)=0,"",IF(L249&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" s="10" t="n"/>
+      <c r="B250" s="11" t="n"/>
+      <c r="C250" s="11" t="n"/>
+      <c r="D250" s="11" t="n"/>
+      <c r="E250" s="11" t="n"/>
+      <c r="F250" s="11" t="n"/>
+      <c r="G250" s="11" t="n"/>
+      <c r="H250" s="11" t="n"/>
+      <c r="I250" s="11" t="n"/>
+      <c r="J250" s="12" t="n"/>
+      <c r="K250" s="12" t="n"/>
+      <c r="L250" s="13">
+        <f>COUNTIF(E250:G250,"有")+IF(H250&gt;=6,1,0)+IF(I250&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M250" s="11" t="n"/>
+      <c r="N250" s="13">
+        <f>IF(COUNTA(A250:G250)=0,"",IF(L250&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" s="10" t="n"/>
+      <c r="B251" s="11" t="n"/>
+      <c r="C251" s="11" t="n"/>
+      <c r="D251" s="11" t="n"/>
+      <c r="E251" s="11" t="n"/>
+      <c r="F251" s="11" t="n"/>
+      <c r="G251" s="11" t="n"/>
+      <c r="H251" s="11" t="n"/>
+      <c r="I251" s="11" t="n"/>
+      <c r="J251" s="12" t="n"/>
+      <c r="K251" s="12" t="n"/>
+      <c r="L251" s="13">
+        <f>COUNTIF(E251:G251,"有")+IF(H251&gt;=6,1,0)+IF(I251&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M251" s="11" t="n"/>
+      <c r="N251" s="13">
+        <f>IF(COUNTA(A251:G251)=0,"",IF(L251&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" s="10" t="n"/>
+      <c r="B252" s="11" t="n"/>
+      <c r="C252" s="11" t="n"/>
+      <c r="D252" s="11" t="n"/>
+      <c r="E252" s="11" t="n"/>
+      <c r="F252" s="11" t="n"/>
+      <c r="G252" s="11" t="n"/>
+      <c r="H252" s="11" t="n"/>
+      <c r="I252" s="11" t="n"/>
+      <c r="J252" s="12" t="n"/>
+      <c r="K252" s="12" t="n"/>
+      <c r="L252" s="13">
+        <f>COUNTIF(E252:G252,"有")+IF(H252&gt;=6,1,0)+IF(I252&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M252" s="11" t="n"/>
+      <c r="N252" s="13">
+        <f>IF(COUNTA(A252:G252)=0,"",IF(L252&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" s="10" t="n"/>
+      <c r="B253" s="11" t="n"/>
+      <c r="C253" s="11" t="n"/>
+      <c r="D253" s="11" t="n"/>
+      <c r="E253" s="11" t="n"/>
+      <c r="F253" s="11" t="n"/>
+      <c r="G253" s="11" t="n"/>
+      <c r="H253" s="11" t="n"/>
+      <c r="I253" s="11" t="n"/>
+      <c r="J253" s="12" t="n"/>
+      <c r="K253" s="12" t="n"/>
+      <c r="L253" s="13">
+        <f>COUNTIF(E253:G253,"有")+IF(H253&gt;=6,1,0)+IF(I253&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M253" s="11" t="n"/>
+      <c r="N253" s="13">
+        <f>IF(COUNTA(A253:G253)=0,"",IF(L253&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" s="10" t="n"/>
+      <c r="B254" s="11" t="n"/>
+      <c r="C254" s="11" t="n"/>
+      <c r="D254" s="11" t="n"/>
+      <c r="E254" s="11" t="n"/>
+      <c r="F254" s="11" t="n"/>
+      <c r="G254" s="11" t="n"/>
+      <c r="H254" s="11" t="n"/>
+      <c r="I254" s="11" t="n"/>
+      <c r="J254" s="12" t="n"/>
+      <c r="K254" s="12" t="n"/>
+      <c r="L254" s="13">
+        <f>COUNTIF(E254:G254,"有")+IF(H254&gt;=6,1,0)+IF(I254&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M254" s="11" t="n"/>
+      <c r="N254" s="13">
+        <f>IF(COUNTA(A254:G254)=0,"",IF(L254&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" s="10" t="n"/>
+      <c r="B255" s="11" t="n"/>
+      <c r="C255" s="11" t="n"/>
+      <c r="D255" s="11" t="n"/>
+      <c r="E255" s="11" t="n"/>
+      <c r="F255" s="11" t="n"/>
+      <c r="G255" s="11" t="n"/>
+      <c r="H255" s="11" t="n"/>
+      <c r="I255" s="11" t="n"/>
+      <c r="J255" s="12" t="n"/>
+      <c r="K255" s="12" t="n"/>
+      <c r="L255" s="13">
+        <f>COUNTIF(E255:G255,"有")+IF(H255&gt;=6,1,0)+IF(I255&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M255" s="11" t="n"/>
+      <c r="N255" s="13">
+        <f>IF(COUNTA(A255:G255)=0,"",IF(L255&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" s="10" t="n"/>
+      <c r="B256" s="11" t="n"/>
+      <c r="C256" s="11" t="n"/>
+      <c r="D256" s="11" t="n"/>
+      <c r="E256" s="11" t="n"/>
+      <c r="F256" s="11" t="n"/>
+      <c r="G256" s="11" t="n"/>
+      <c r="H256" s="11" t="n"/>
+      <c r="I256" s="11" t="n"/>
+      <c r="J256" s="12" t="n"/>
+      <c r="K256" s="12" t="n"/>
+      <c r="L256" s="13">
+        <f>COUNTIF(E256:G256,"有")+IF(H256&gt;=6,1,0)+IF(I256&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M256" s="11" t="n"/>
+      <c r="N256" s="13">
+        <f>IF(COUNTA(A256:G256)=0,"",IF(L256&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" s="10" t="n"/>
+      <c r="B257" s="11" t="n"/>
+      <c r="C257" s="11" t="n"/>
+      <c r="D257" s="11" t="n"/>
+      <c r="E257" s="11" t="n"/>
+      <c r="F257" s="11" t="n"/>
+      <c r="G257" s="11" t="n"/>
+      <c r="H257" s="11" t="n"/>
+      <c r="I257" s="11" t="n"/>
+      <c r="J257" s="12" t="n"/>
+      <c r="K257" s="12" t="n"/>
+      <c r="L257" s="13">
+        <f>COUNTIF(E257:G257,"有")+IF(H257&gt;=6,1,0)+IF(I257&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M257" s="11" t="n"/>
+      <c r="N257" s="13">
+        <f>IF(COUNTA(A257:G257)=0,"",IF(L257&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" s="10" t="n"/>
+      <c r="B258" s="11" t="n"/>
+      <c r="C258" s="11" t="n"/>
+      <c r="D258" s="11" t="n"/>
+      <c r="E258" s="11" t="n"/>
+      <c r="F258" s="11" t="n"/>
+      <c r="G258" s="11" t="n"/>
+      <c r="H258" s="11" t="n"/>
+      <c r="I258" s="11" t="n"/>
+      <c r="J258" s="12" t="n"/>
+      <c r="K258" s="12" t="n"/>
+      <c r="L258" s="13">
+        <f>COUNTIF(E258:G258,"有")+IF(H258&gt;=6,1,0)+IF(I258&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M258" s="11" t="n"/>
+      <c r="N258" s="13">
+        <f>IF(COUNTA(A258:G258)=0,"",IF(L258&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" s="10" t="n"/>
+      <c r="B259" s="11" t="n"/>
+      <c r="C259" s="11" t="n"/>
+      <c r="D259" s="11" t="n"/>
+      <c r="E259" s="11" t="n"/>
+      <c r="F259" s="11" t="n"/>
+      <c r="G259" s="11" t="n"/>
+      <c r="H259" s="11" t="n"/>
+      <c r="I259" s="11" t="n"/>
+      <c r="J259" s="12" t="n"/>
+      <c r="K259" s="12" t="n"/>
+      <c r="L259" s="13">
+        <f>COUNTIF(E259:G259,"有")+IF(H259&gt;=6,1,0)+IF(I259&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M259" s="11" t="n"/>
+      <c r="N259" s="13">
+        <f>IF(COUNTA(A259:G259)=0,"",IF(L259&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" s="10" t="n"/>
+      <c r="B260" s="11" t="n"/>
+      <c r="C260" s="11" t="n"/>
+      <c r="D260" s="11" t="n"/>
+      <c r="E260" s="11" t="n"/>
+      <c r="F260" s="11" t="n"/>
+      <c r="G260" s="11" t="n"/>
+      <c r="H260" s="11" t="n"/>
+      <c r="I260" s="11" t="n"/>
+      <c r="J260" s="12" t="n"/>
+      <c r="K260" s="12" t="n"/>
+      <c r="L260" s="13">
+        <f>COUNTIF(E260:G260,"有")+IF(H260&gt;=6,1,0)+IF(I260&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M260" s="11" t="n"/>
+      <c r="N260" s="13">
+        <f>IF(COUNTA(A260:G260)=0,"",IF(L260&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" s="10" t="n"/>
+      <c r="B261" s="11" t="n"/>
+      <c r="C261" s="11" t="n"/>
+      <c r="D261" s="11" t="n"/>
+      <c r="E261" s="11" t="n"/>
+      <c r="F261" s="11" t="n"/>
+      <c r="G261" s="11" t="n"/>
+      <c r="H261" s="11" t="n"/>
+      <c r="I261" s="11" t="n"/>
+      <c r="J261" s="12" t="n"/>
+      <c r="K261" s="12" t="n"/>
+      <c r="L261" s="13">
+        <f>COUNTIF(E261:G261,"有")+IF(H261&gt;=6,1,0)+IF(I261&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M261" s="11" t="n"/>
+      <c r="N261" s="13">
+        <f>IF(COUNTA(A261:G261)=0,"",IF(L261&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" s="10" t="n"/>
+      <c r="B262" s="11" t="n"/>
+      <c r="C262" s="11" t="n"/>
+      <c r="D262" s="11" t="n"/>
+      <c r="E262" s="11" t="n"/>
+      <c r="F262" s="11" t="n"/>
+      <c r="G262" s="11" t="n"/>
+      <c r="H262" s="11" t="n"/>
+      <c r="I262" s="11" t="n"/>
+      <c r="J262" s="12" t="n"/>
+      <c r="K262" s="12" t="n"/>
+      <c r="L262" s="13">
+        <f>COUNTIF(E262:G262,"有")+IF(H262&gt;=6,1,0)+IF(I262&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M262" s="11" t="n"/>
+      <c r="N262" s="13">
+        <f>IF(COUNTA(A262:G262)=0,"",IF(L262&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" s="10" t="n"/>
+      <c r="B263" s="11" t="n"/>
+      <c r="C263" s="11" t="n"/>
+      <c r="D263" s="11" t="n"/>
+      <c r="E263" s="11" t="n"/>
+      <c r="F263" s="11" t="n"/>
+      <c r="G263" s="11" t="n"/>
+      <c r="H263" s="11" t="n"/>
+      <c r="I263" s="11" t="n"/>
+      <c r="J263" s="12" t="n"/>
+      <c r="K263" s="12" t="n"/>
+      <c r="L263" s="13">
+        <f>COUNTIF(E263:G263,"有")+IF(H263&gt;=6,1,0)+IF(I263&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M263" s="11" t="n"/>
+      <c r="N263" s="13">
+        <f>IF(COUNTA(A263:G263)=0,"",IF(L263&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="10" t="n"/>
+      <c r="B264" s="11" t="n"/>
+      <c r="C264" s="11" t="n"/>
+      <c r="D264" s="11" t="n"/>
+      <c r="E264" s="11" t="n"/>
+      <c r="F264" s="11" t="n"/>
+      <c r="G264" s="11" t="n"/>
+      <c r="H264" s="11" t="n"/>
+      <c r="I264" s="11" t="n"/>
+      <c r="J264" s="12" t="n"/>
+      <c r="K264" s="12" t="n"/>
+      <c r="L264" s="13">
+        <f>COUNTIF(E264:G264,"有")+IF(H264&gt;=6,1,0)+IF(I264&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M264" s="11" t="n"/>
+      <c r="N264" s="13">
+        <f>IF(COUNTA(A264:G264)=0,"",IF(L264&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" s="10" t="n"/>
+      <c r="B265" s="11" t="n"/>
+      <c r="C265" s="11" t="n"/>
+      <c r="D265" s="11" t="n"/>
+      <c r="E265" s="11" t="n"/>
+      <c r="F265" s="11" t="n"/>
+      <c r="G265" s="11" t="n"/>
+      <c r="H265" s="11" t="n"/>
+      <c r="I265" s="11" t="n"/>
+      <c r="J265" s="12" t="n"/>
+      <c r="K265" s="12" t="n"/>
+      <c r="L265" s="13">
+        <f>COUNTIF(E265:G265,"有")+IF(H265&gt;=6,1,0)+IF(I265&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M265" s="11" t="n"/>
+      <c r="N265" s="13">
+        <f>IF(COUNTA(A265:G265)=0,"",IF(L265&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" s="10" t="n"/>
+      <c r="B266" s="11" t="n"/>
+      <c r="C266" s="11" t="n"/>
+      <c r="D266" s="11" t="n"/>
+      <c r="E266" s="11" t="n"/>
+      <c r="F266" s="11" t="n"/>
+      <c r="G266" s="11" t="n"/>
+      <c r="H266" s="11" t="n"/>
+      <c r="I266" s="11" t="n"/>
+      <c r="J266" s="12" t="n"/>
+      <c r="K266" s="12" t="n"/>
+      <c r="L266" s="13">
+        <f>COUNTIF(E266:G266,"有")+IF(H266&gt;=6,1,0)+IF(I266&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M266" s="11" t="n"/>
+      <c r="N266" s="13">
+        <f>IF(COUNTA(A266:G266)=0,"",IF(L266&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" s="10" t="n"/>
+      <c r="B267" s="11" t="n"/>
+      <c r="C267" s="11" t="n"/>
+      <c r="D267" s="11" t="n"/>
+      <c r="E267" s="11" t="n"/>
+      <c r="F267" s="11" t="n"/>
+      <c r="G267" s="11" t="n"/>
+      <c r="H267" s="11" t="n"/>
+      <c r="I267" s="11" t="n"/>
+      <c r="J267" s="12" t="n"/>
+      <c r="K267" s="12" t="n"/>
+      <c r="L267" s="13">
+        <f>COUNTIF(E267:G267,"有")+IF(H267&gt;=6,1,0)+IF(I267&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M267" s="11" t="n"/>
+      <c r="N267" s="13">
+        <f>IF(COUNTA(A267:G267)=0,"",IF(L267&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" s="10" t="n"/>
+      <c r="B268" s="11" t="n"/>
+      <c r="C268" s="11" t="n"/>
+      <c r="D268" s="11" t="n"/>
+      <c r="E268" s="11" t="n"/>
+      <c r="F268" s="11" t="n"/>
+      <c r="G268" s="11" t="n"/>
+      <c r="H268" s="11" t="n"/>
+      <c r="I268" s="11" t="n"/>
+      <c r="J268" s="12" t="n"/>
+      <c r="K268" s="12" t="n"/>
+      <c r="L268" s="13">
+        <f>COUNTIF(E268:G268,"有")+IF(H268&gt;=6,1,0)+IF(I268&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M268" s="11" t="n"/>
+      <c r="N268" s="13">
+        <f>IF(COUNTA(A268:G268)=0,"",IF(L268&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" s="10" t="n"/>
+      <c r="B269" s="11" t="n"/>
+      <c r="C269" s="11" t="n"/>
+      <c r="D269" s="11" t="n"/>
+      <c r="E269" s="11" t="n"/>
+      <c r="F269" s="11" t="n"/>
+      <c r="G269" s="11" t="n"/>
+      <c r="H269" s="11" t="n"/>
+      <c r="I269" s="11" t="n"/>
+      <c r="J269" s="12" t="n"/>
+      <c r="K269" s="12" t="n"/>
+      <c r="L269" s="13">
+        <f>COUNTIF(E269:G269,"有")+IF(H269&gt;=6,1,0)+IF(I269&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M269" s="11" t="n"/>
+      <c r="N269" s="13">
+        <f>IF(COUNTA(A269:G269)=0,"",IF(L269&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" s="10" t="n"/>
+      <c r="B270" s="11" t="n"/>
+      <c r="C270" s="11" t="n"/>
+      <c r="D270" s="11" t="n"/>
+      <c r="E270" s="11" t="n"/>
+      <c r="F270" s="11" t="n"/>
+      <c r="G270" s="11" t="n"/>
+      <c r="H270" s="11" t="n"/>
+      <c r="I270" s="11" t="n"/>
+      <c r="J270" s="12" t="n"/>
+      <c r="K270" s="12" t="n"/>
+      <c r="L270" s="13">
+        <f>COUNTIF(E270:G270,"有")+IF(H270&gt;=6,1,0)+IF(I270&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M270" s="11" t="n"/>
+      <c r="N270" s="13">
+        <f>IF(COUNTA(A270:G270)=0,"",IF(L270&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" s="10" t="n"/>
+      <c r="B271" s="11" t="n"/>
+      <c r="C271" s="11" t="n"/>
+      <c r="D271" s="11" t="n"/>
+      <c r="E271" s="11" t="n"/>
+      <c r="F271" s="11" t="n"/>
+      <c r="G271" s="11" t="n"/>
+      <c r="H271" s="11" t="n"/>
+      <c r="I271" s="11" t="n"/>
+      <c r="J271" s="12" t="n"/>
+      <c r="K271" s="12" t="n"/>
+      <c r="L271" s="13">
+        <f>COUNTIF(E271:G271,"有")+IF(H271&gt;=6,1,0)+IF(I271&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M271" s="11" t="n"/>
+      <c r="N271" s="13">
+        <f>IF(COUNTA(A271:G271)=0,"",IF(L271&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" s="10" t="n"/>
+      <c r="B272" s="11" t="n"/>
+      <c r="C272" s="11" t="n"/>
+      <c r="D272" s="11" t="n"/>
+      <c r="E272" s="11" t="n"/>
+      <c r="F272" s="11" t="n"/>
+      <c r="G272" s="11" t="n"/>
+      <c r="H272" s="11" t="n"/>
+      <c r="I272" s="11" t="n"/>
+      <c r="J272" s="12" t="n"/>
+      <c r="K272" s="12" t="n"/>
+      <c r="L272" s="13">
+        <f>COUNTIF(E272:G272,"有")+IF(H272&gt;=6,1,0)+IF(I272&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M272" s="11" t="n"/>
+      <c r="N272" s="13">
+        <f>IF(COUNTA(A272:G272)=0,"",IF(L272&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" s="10" t="n"/>
+      <c r="B273" s="11" t="n"/>
+      <c r="C273" s="11" t="n"/>
+      <c r="D273" s="11" t="n"/>
+      <c r="E273" s="11" t="n"/>
+      <c r="F273" s="11" t="n"/>
+      <c r="G273" s="11" t="n"/>
+      <c r="H273" s="11" t="n"/>
+      <c r="I273" s="11" t="n"/>
+      <c r="J273" s="12" t="n"/>
+      <c r="K273" s="12" t="n"/>
+      <c r="L273" s="13">
+        <f>COUNTIF(E273:G273,"有")+IF(H273&gt;=6,1,0)+IF(I273&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M273" s="11" t="n"/>
+      <c r="N273" s="13">
+        <f>IF(COUNTA(A273:G273)=0,"",IF(L273&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" s="10" t="n"/>
+      <c r="B274" s="11" t="n"/>
+      <c r="C274" s="11" t="n"/>
+      <c r="D274" s="11" t="n"/>
+      <c r="E274" s="11" t="n"/>
+      <c r="F274" s="11" t="n"/>
+      <c r="G274" s="11" t="n"/>
+      <c r="H274" s="11" t="n"/>
+      <c r="I274" s="11" t="n"/>
+      <c r="J274" s="12" t="n"/>
+      <c r="K274" s="12" t="n"/>
+      <c r="L274" s="13">
+        <f>COUNTIF(E274:G274,"有")+IF(H274&gt;=6,1,0)+IF(I274&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M274" s="11" t="n"/>
+      <c r="N274" s="13">
+        <f>IF(COUNTA(A274:G274)=0,"",IF(L274&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" s="10" t="n"/>
+      <c r="B275" s="11" t="n"/>
+      <c r="C275" s="11" t="n"/>
+      <c r="D275" s="11" t="n"/>
+      <c r="E275" s="11" t="n"/>
+      <c r="F275" s="11" t="n"/>
+      <c r="G275" s="11" t="n"/>
+      <c r="H275" s="11" t="n"/>
+      <c r="I275" s="11" t="n"/>
+      <c r="J275" s="12" t="n"/>
+      <c r="K275" s="12" t="n"/>
+      <c r="L275" s="13">
+        <f>COUNTIF(E275:G275,"有")+IF(H275&gt;=6,1,0)+IF(I275&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M275" s="11" t="n"/>
+      <c r="N275" s="13">
+        <f>IF(COUNTA(A275:G275)=0,"",IF(L275&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" s="10" t="n"/>
+      <c r="B276" s="11" t="n"/>
+      <c r="C276" s="11" t="n"/>
+      <c r="D276" s="11" t="n"/>
+      <c r="E276" s="11" t="n"/>
+      <c r="F276" s="11" t="n"/>
+      <c r="G276" s="11" t="n"/>
+      <c r="H276" s="11" t="n"/>
+      <c r="I276" s="11" t="n"/>
+      <c r="J276" s="12" t="n"/>
+      <c r="K276" s="12" t="n"/>
+      <c r="L276" s="13">
+        <f>COUNTIF(E276:G276,"有")+IF(H276&gt;=6,1,0)+IF(I276&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M276" s="11" t="n"/>
+      <c r="N276" s="13">
+        <f>IF(COUNTA(A276:G276)=0,"",IF(L276&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" s="10" t="n"/>
+      <c r="B277" s="11" t="n"/>
+      <c r="C277" s="11" t="n"/>
+      <c r="D277" s="11" t="n"/>
+      <c r="E277" s="11" t="n"/>
+      <c r="F277" s="11" t="n"/>
+      <c r="G277" s="11" t="n"/>
+      <c r="H277" s="11" t="n"/>
+      <c r="I277" s="11" t="n"/>
+      <c r="J277" s="12" t="n"/>
+      <c r="K277" s="12" t="n"/>
+      <c r="L277" s="13">
+        <f>COUNTIF(E277:G277,"有")+IF(H277&gt;=6,1,0)+IF(I277&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M277" s="11" t="n"/>
+      <c r="N277" s="13">
+        <f>IF(COUNTA(A277:G277)=0,"",IF(L277&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" s="10" t="n"/>
+      <c r="B278" s="11" t="n"/>
+      <c r="C278" s="11" t="n"/>
+      <c r="D278" s="11" t="n"/>
+      <c r="E278" s="11" t="n"/>
+      <c r="F278" s="11" t="n"/>
+      <c r="G278" s="11" t="n"/>
+      <c r="H278" s="11" t="n"/>
+      <c r="I278" s="11" t="n"/>
+      <c r="J278" s="12" t="n"/>
+      <c r="K278" s="12" t="n"/>
+      <c r="L278" s="13">
+        <f>COUNTIF(E278:G278,"有")+IF(H278&gt;=6,1,0)+IF(I278&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M278" s="11" t="n"/>
+      <c r="N278" s="13">
+        <f>IF(COUNTA(A278:G278)=0,"",IF(L278&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" s="10" t="n"/>
+      <c r="B279" s="11" t="n"/>
+      <c r="C279" s="11" t="n"/>
+      <c r="D279" s="11" t="n"/>
+      <c r="E279" s="11" t="n"/>
+      <c r="F279" s="11" t="n"/>
+      <c r="G279" s="11" t="n"/>
+      <c r="H279" s="11" t="n"/>
+      <c r="I279" s="11" t="n"/>
+      <c r="J279" s="12" t="n"/>
+      <c r="K279" s="12" t="n"/>
+      <c r="L279" s="13">
+        <f>COUNTIF(E279:G279,"有")+IF(H279&gt;=6,1,0)+IF(I279&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M279" s="11" t="n"/>
+      <c r="N279" s="13">
+        <f>IF(COUNTA(A279:G279)=0,"",IF(L279&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" s="10" t="n"/>
+      <c r="B280" s="11" t="n"/>
+      <c r="C280" s="11" t="n"/>
+      <c r="D280" s="11" t="n"/>
+      <c r="E280" s="11" t="n"/>
+      <c r="F280" s="11" t="n"/>
+      <c r="G280" s="11" t="n"/>
+      <c r="H280" s="11" t="n"/>
+      <c r="I280" s="11" t="n"/>
+      <c r="J280" s="12" t="n"/>
+      <c r="K280" s="12" t="n"/>
+      <c r="L280" s="13">
+        <f>COUNTIF(E280:G280,"有")+IF(H280&gt;=6,1,0)+IF(I280&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M280" s="11" t="n"/>
+      <c r="N280" s="13">
+        <f>IF(COUNTA(A280:G280)=0,"",IF(L280&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" s="10" t="n"/>
+      <c r="B281" s="11" t="n"/>
+      <c r="C281" s="11" t="n"/>
+      <c r="D281" s="11" t="n"/>
+      <c r="E281" s="11" t="n"/>
+      <c r="F281" s="11" t="n"/>
+      <c r="G281" s="11" t="n"/>
+      <c r="H281" s="11" t="n"/>
+      <c r="I281" s="11" t="n"/>
+      <c r="J281" s="12" t="n"/>
+      <c r="K281" s="12" t="n"/>
+      <c r="L281" s="13">
+        <f>COUNTIF(E281:G281,"有")+IF(H281&gt;=6,1,0)+IF(I281&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M281" s="11" t="n"/>
+      <c r="N281" s="13">
+        <f>IF(COUNTA(A281:G281)=0,"",IF(L281&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" s="10" t="n"/>
+      <c r="B282" s="11" t="n"/>
+      <c r="C282" s="11" t="n"/>
+      <c r="D282" s="11" t="n"/>
+      <c r="E282" s="11" t="n"/>
+      <c r="F282" s="11" t="n"/>
+      <c r="G282" s="11" t="n"/>
+      <c r="H282" s="11" t="n"/>
+      <c r="I282" s="11" t="n"/>
+      <c r="J282" s="12" t="n"/>
+      <c r="K282" s="12" t="n"/>
+      <c r="L282" s="13">
+        <f>COUNTIF(E282:G282,"有")+IF(H282&gt;=6,1,0)+IF(I282&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M282" s="11" t="n"/>
+      <c r="N282" s="13">
+        <f>IF(COUNTA(A282:G282)=0,"",IF(L282&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" s="10" t="n"/>
+      <c r="B283" s="11" t="n"/>
+      <c r="C283" s="11" t="n"/>
+      <c r="D283" s="11" t="n"/>
+      <c r="E283" s="11" t="n"/>
+      <c r="F283" s="11" t="n"/>
+      <c r="G283" s="11" t="n"/>
+      <c r="H283" s="11" t="n"/>
+      <c r="I283" s="11" t="n"/>
+      <c r="J283" s="12" t="n"/>
+      <c r="K283" s="12" t="n"/>
+      <c r="L283" s="13">
+        <f>COUNTIF(E283:G283,"有")+IF(H283&gt;=6,1,0)+IF(I283&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M283" s="11" t="n"/>
+      <c r="N283" s="13">
+        <f>IF(COUNTA(A283:G283)=0,"",IF(L283&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" s="10" t="n"/>
+      <c r="B284" s="11" t="n"/>
+      <c r="C284" s="11" t="n"/>
+      <c r="D284" s="11" t="n"/>
+      <c r="E284" s="11" t="n"/>
+      <c r="F284" s="11" t="n"/>
+      <c r="G284" s="11" t="n"/>
+      <c r="H284" s="11" t="n"/>
+      <c r="I284" s="11" t="n"/>
+      <c r="J284" s="12" t="n"/>
+      <c r="K284" s="12" t="n"/>
+      <c r="L284" s="13">
+        <f>COUNTIF(E284:G284,"有")+IF(H284&gt;=6,1,0)+IF(I284&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M284" s="11" t="n"/>
+      <c r="N284" s="13">
+        <f>IF(COUNTA(A284:G284)=0,"",IF(L284&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" s="10" t="n"/>
+      <c r="B285" s="11" t="n"/>
+      <c r="C285" s="11" t="n"/>
+      <c r="D285" s="11" t="n"/>
+      <c r="E285" s="11" t="n"/>
+      <c r="F285" s="11" t="n"/>
+      <c r="G285" s="11" t="n"/>
+      <c r="H285" s="11" t="n"/>
+      <c r="I285" s="11" t="n"/>
+      <c r="J285" s="12" t="n"/>
+      <c r="K285" s="12" t="n"/>
+      <c r="L285" s="13">
+        <f>COUNTIF(E285:G285,"有")+IF(H285&gt;=6,1,0)+IF(I285&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M285" s="11" t="n"/>
+      <c r="N285" s="13">
+        <f>IF(COUNTA(A285:G285)=0,"",IF(L285&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" s="10" t="n"/>
+      <c r="B286" s="11" t="n"/>
+      <c r="C286" s="11" t="n"/>
+      <c r="D286" s="11" t="n"/>
+      <c r="E286" s="11" t="n"/>
+      <c r="F286" s="11" t="n"/>
+      <c r="G286" s="11" t="n"/>
+      <c r="H286" s="11" t="n"/>
+      <c r="I286" s="11" t="n"/>
+      <c r="J286" s="12" t="n"/>
+      <c r="K286" s="12" t="n"/>
+      <c r="L286" s="13">
+        <f>COUNTIF(E286:G286,"有")+IF(H286&gt;=6,1,0)+IF(I286&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M286" s="11" t="n"/>
+      <c r="N286" s="13">
+        <f>IF(COUNTA(A286:G286)=0,"",IF(L286&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" s="10" t="n"/>
+      <c r="B287" s="11" t="n"/>
+      <c r="C287" s="11" t="n"/>
+      <c r="D287" s="11" t="n"/>
+      <c r="E287" s="11" t="n"/>
+      <c r="F287" s="11" t="n"/>
+      <c r="G287" s="11" t="n"/>
+      <c r="H287" s="11" t="n"/>
+      <c r="I287" s="11" t="n"/>
+      <c r="J287" s="12" t="n"/>
+      <c r="K287" s="12" t="n"/>
+      <c r="L287" s="13">
+        <f>COUNTIF(E287:G287,"有")+IF(H287&gt;=6,1,0)+IF(I287&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M287" s="11" t="n"/>
+      <c r="N287" s="13">
+        <f>IF(COUNTA(A287:G287)=0,"",IF(L287&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" s="10" t="n"/>
+      <c r="B288" s="11" t="n"/>
+      <c r="C288" s="11" t="n"/>
+      <c r="D288" s="11" t="n"/>
+      <c r="E288" s="11" t="n"/>
+      <c r="F288" s="11" t="n"/>
+      <c r="G288" s="11" t="n"/>
+      <c r="H288" s="11" t="n"/>
+      <c r="I288" s="11" t="n"/>
+      <c r="J288" s="12" t="n"/>
+      <c r="K288" s="12" t="n"/>
+      <c r="L288" s="13">
+        <f>COUNTIF(E288:G288,"有")+IF(H288&gt;=6,1,0)+IF(I288&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M288" s="11" t="n"/>
+      <c r="N288" s="13">
+        <f>IF(COUNTA(A288:G288)=0,"",IF(L288&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" s="10" t="n"/>
+      <c r="B289" s="11" t="n"/>
+      <c r="C289" s="11" t="n"/>
+      <c r="D289" s="11" t="n"/>
+      <c r="E289" s="11" t="n"/>
+      <c r="F289" s="11" t="n"/>
+      <c r="G289" s="11" t="n"/>
+      <c r="H289" s="11" t="n"/>
+      <c r="I289" s="11" t="n"/>
+      <c r="J289" s="12" t="n"/>
+      <c r="K289" s="12" t="n"/>
+      <c r="L289" s="13">
+        <f>COUNTIF(E289:G289,"有")+IF(H289&gt;=6,1,0)+IF(I289&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M289" s="11" t="n"/>
+      <c r="N289" s="13">
+        <f>IF(COUNTA(A289:G289)=0,"",IF(L289&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" s="10" t="n"/>
+      <c r="B290" s="11" t="n"/>
+      <c r="C290" s="11" t="n"/>
+      <c r="D290" s="11" t="n"/>
+      <c r="E290" s="11" t="n"/>
+      <c r="F290" s="11" t="n"/>
+      <c r="G290" s="11" t="n"/>
+      <c r="H290" s="11" t="n"/>
+      <c r="I290" s="11" t="n"/>
+      <c r="J290" s="12" t="n"/>
+      <c r="K290" s="12" t="n"/>
+      <c r="L290" s="13">
+        <f>COUNTIF(E290:G290,"有")+IF(H290&gt;=6,1,0)+IF(I290&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M290" s="11" t="n"/>
+      <c r="N290" s="13">
+        <f>IF(COUNTA(A290:G290)=0,"",IF(L290&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" s="10" t="n"/>
+      <c r="B291" s="11" t="n"/>
+      <c r="C291" s="11" t="n"/>
+      <c r="D291" s="11" t="n"/>
+      <c r="E291" s="11" t="n"/>
+      <c r="F291" s="11" t="n"/>
+      <c r="G291" s="11" t="n"/>
+      <c r="H291" s="11" t="n"/>
+      <c r="I291" s="11" t="n"/>
+      <c r="J291" s="12" t="n"/>
+      <c r="K291" s="12" t="n"/>
+      <c r="L291" s="13">
+        <f>COUNTIF(E291:G291,"有")+IF(H291&gt;=6,1,0)+IF(I291&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M291" s="11" t="n"/>
+      <c r="N291" s="13">
+        <f>IF(COUNTA(A291:G291)=0,"",IF(L291&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" s="10" t="n"/>
+      <c r="B292" s="11" t="n"/>
+      <c r="C292" s="11" t="n"/>
+      <c r="D292" s="11" t="n"/>
+      <c r="E292" s="11" t="n"/>
+      <c r="F292" s="11" t="n"/>
+      <c r="G292" s="11" t="n"/>
+      <c r="H292" s="11" t="n"/>
+      <c r="I292" s="11" t="n"/>
+      <c r="J292" s="12" t="n"/>
+      <c r="K292" s="12" t="n"/>
+      <c r="L292" s="13">
+        <f>COUNTIF(E292:G292,"有")+IF(H292&gt;=6,1,0)+IF(I292&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M292" s="11" t="n"/>
+      <c r="N292" s="13">
+        <f>IF(COUNTA(A292:G292)=0,"",IF(L292&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" s="10" t="n"/>
+      <c r="B293" s="11" t="n"/>
+      <c r="C293" s="11" t="n"/>
+      <c r="D293" s="11" t="n"/>
+      <c r="E293" s="11" t="n"/>
+      <c r="F293" s="11" t="n"/>
+      <c r="G293" s="11" t="n"/>
+      <c r="H293" s="11" t="n"/>
+      <c r="I293" s="11" t="n"/>
+      <c r="J293" s="12" t="n"/>
+      <c r="K293" s="12" t="n"/>
+      <c r="L293" s="13">
+        <f>COUNTIF(E293:G293,"有")+IF(H293&gt;=6,1,0)+IF(I293&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M293" s="11" t="n"/>
+      <c r="N293" s="13">
+        <f>IF(COUNTA(A293:G293)=0,"",IF(L293&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" s="10" t="n"/>
+      <c r="B294" s="11" t="n"/>
+      <c r="C294" s="11" t="n"/>
+      <c r="D294" s="11" t="n"/>
+      <c r="E294" s="11" t="n"/>
+      <c r="F294" s="11" t="n"/>
+      <c r="G294" s="11" t="n"/>
+      <c r="H294" s="11" t="n"/>
+      <c r="I294" s="11" t="n"/>
+      <c r="J294" s="12" t="n"/>
+      <c r="K294" s="12" t="n"/>
+      <c r="L294" s="13">
+        <f>COUNTIF(E294:G294,"有")+IF(H294&gt;=6,1,0)+IF(I294&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M294" s="11" t="n"/>
+      <c r="N294" s="13">
+        <f>IF(COUNTA(A294:G294)=0,"",IF(L294&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" s="10" t="n"/>
+      <c r="B295" s="11" t="n"/>
+      <c r="C295" s="11" t="n"/>
+      <c r="D295" s="11" t="n"/>
+      <c r="E295" s="11" t="n"/>
+      <c r="F295" s="11" t="n"/>
+      <c r="G295" s="11" t="n"/>
+      <c r="H295" s="11" t="n"/>
+      <c r="I295" s="11" t="n"/>
+      <c r="J295" s="12" t="n"/>
+      <c r="K295" s="12" t="n"/>
+      <c r="L295" s="13">
+        <f>COUNTIF(E295:G295,"有")+IF(H295&gt;=6,1,0)+IF(I295&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M295" s="11" t="n"/>
+      <c r="N295" s="13">
+        <f>IF(COUNTA(A295:G295)=0,"",IF(L295&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" s="10" t="n"/>
+      <c r="B296" s="11" t="n"/>
+      <c r="C296" s="11" t="n"/>
+      <c r="D296" s="11" t="n"/>
+      <c r="E296" s="11" t="n"/>
+      <c r="F296" s="11" t="n"/>
+      <c r="G296" s="11" t="n"/>
+      <c r="H296" s="11" t="n"/>
+      <c r="I296" s="11" t="n"/>
+      <c r="J296" s="12" t="n"/>
+      <c r="K296" s="12" t="n"/>
+      <c r="L296" s="13">
+        <f>COUNTIF(E296:G296,"有")+IF(H296&gt;=6,1,0)+IF(I296&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M296" s="11" t="n"/>
+      <c r="N296" s="13">
+        <f>IF(COUNTA(A296:G296)=0,"",IF(L296&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" s="10" t="n"/>
+      <c r="B297" s="11" t="n"/>
+      <c r="C297" s="11" t="n"/>
+      <c r="D297" s="11" t="n"/>
+      <c r="E297" s="11" t="n"/>
+      <c r="F297" s="11" t="n"/>
+      <c r="G297" s="11" t="n"/>
+      <c r="H297" s="11" t="n"/>
+      <c r="I297" s="11" t="n"/>
+      <c r="J297" s="12" t="n"/>
+      <c r="K297" s="12" t="n"/>
+      <c r="L297" s="13">
+        <f>COUNTIF(E297:G297,"有")+IF(H297&gt;=6,1,0)+IF(I297&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M297" s="11" t="n"/>
+      <c r="N297" s="13">
+        <f>IF(COUNTA(A297:G297)=0,"",IF(L297&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" s="10" t="n"/>
+      <c r="B298" s="11" t="n"/>
+      <c r="C298" s="11" t="n"/>
+      <c r="D298" s="11" t="n"/>
+      <c r="E298" s="11" t="n"/>
+      <c r="F298" s="11" t="n"/>
+      <c r="G298" s="11" t="n"/>
+      <c r="H298" s="11" t="n"/>
+      <c r="I298" s="11" t="n"/>
+      <c r="J298" s="12" t="n"/>
+      <c r="K298" s="12" t="n"/>
+      <c r="L298" s="13">
+        <f>COUNTIF(E298:G298,"有")+IF(H298&gt;=6,1,0)+IF(I298&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M298" s="11" t="n"/>
+      <c r="N298" s="13">
+        <f>IF(COUNTA(A298:G298)=0,"",IF(L298&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" s="10" t="n"/>
+      <c r="B299" s="11" t="n"/>
+      <c r="C299" s="11" t="n"/>
+      <c r="D299" s="11" t="n"/>
+      <c r="E299" s="11" t="n"/>
+      <c r="F299" s="11" t="n"/>
+      <c r="G299" s="11" t="n"/>
+      <c r="H299" s="11" t="n"/>
+      <c r="I299" s="11" t="n"/>
+      <c r="J299" s="12" t="n"/>
+      <c r="K299" s="12" t="n"/>
+      <c r="L299" s="13">
+        <f>COUNTIF(E299:G299,"有")+IF(H299&gt;=6,1,0)+IF(I299&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M299" s="11" t="n"/>
+      <c r="N299" s="13">
+        <f>IF(COUNTA(A299:G299)=0,"",IF(L299&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" s="10" t="n"/>
+      <c r="B300" s="11" t="n"/>
+      <c r="C300" s="11" t="n"/>
+      <c r="D300" s="11" t="n"/>
+      <c r="E300" s="11" t="n"/>
+      <c r="F300" s="11" t="n"/>
+      <c r="G300" s="11" t="n"/>
+      <c r="H300" s="11" t="n"/>
+      <c r="I300" s="11" t="n"/>
+      <c r="J300" s="12" t="n"/>
+      <c r="K300" s="12" t="n"/>
+      <c r="L300" s="13">
+        <f>COUNTIF(E300:G300,"有")+IF(H300&gt;=6,1,0)+IF(I300&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M300" s="11" t="n"/>
+      <c r="N300" s="13">
+        <f>IF(COUNTA(A300:G300)=0,"",IF(L300&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" s="10" t="n"/>
+      <c r="B301" s="11" t="n"/>
+      <c r="C301" s="11" t="n"/>
+      <c r="D301" s="11" t="n"/>
+      <c r="E301" s="11" t="n"/>
+      <c r="F301" s="11" t="n"/>
+      <c r="G301" s="11" t="n"/>
+      <c r="H301" s="11" t="n"/>
+      <c r="I301" s="11" t="n"/>
+      <c r="J301" s="12" t="n"/>
+      <c r="K301" s="12" t="n"/>
+      <c r="L301" s="13">
+        <f>COUNTIF(E301:G301,"有")+IF(H301&gt;=6,1,0)+IF(I301&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M301" s="11" t="n"/>
+      <c r="N301" s="13">
+        <f>IF(COUNTA(A301:G301)=0,"",IF(L301&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" s="10" t="n"/>
+      <c r="B302" s="11" t="n"/>
+      <c r="C302" s="11" t="n"/>
+      <c r="D302" s="11" t="n"/>
+      <c r="E302" s="11" t="n"/>
+      <c r="F302" s="11" t="n"/>
+      <c r="G302" s="11" t="n"/>
+      <c r="H302" s="11" t="n"/>
+      <c r="I302" s="11" t="n"/>
+      <c r="J302" s="12" t="n"/>
+      <c r="K302" s="12" t="n"/>
+      <c r="L302" s="13">
+        <f>COUNTIF(E302:G302,"有")+IF(H302&gt;=6,1,0)+IF(I302&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M302" s="11" t="n"/>
+      <c r="N302" s="13">
+        <f>IF(COUNTA(A302:G302)=0,"",IF(L302&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" s="10" t="n"/>
+      <c r="B303" s="11" t="n"/>
+      <c r="C303" s="11" t="n"/>
+      <c r="D303" s="11" t="n"/>
+      <c r="E303" s="11" t="n"/>
+      <c r="F303" s="11" t="n"/>
+      <c r="G303" s="11" t="n"/>
+      <c r="H303" s="11" t="n"/>
+      <c r="I303" s="11" t="n"/>
+      <c r="J303" s="12" t="n"/>
+      <c r="K303" s="12" t="n"/>
+      <c r="L303" s="13">
+        <f>COUNTIF(E303:G303,"有")+IF(H303&gt;=6,1,0)+IF(I303&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M303" s="11" t="n"/>
+      <c r="N303" s="13">
+        <f>IF(COUNTA(A303:G303)=0,"",IF(L303&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" s="10" t="n"/>
+      <c r="B304" s="11" t="n"/>
+      <c r="C304" s="11" t="n"/>
+      <c r="D304" s="11" t="n"/>
+      <c r="E304" s="11" t="n"/>
+      <c r="F304" s="11" t="n"/>
+      <c r="G304" s="11" t="n"/>
+      <c r="H304" s="11" t="n"/>
+      <c r="I304" s="11" t="n"/>
+      <c r="J304" s="12" t="n"/>
+      <c r="K304" s="12" t="n"/>
+      <c r="L304" s="13">
+        <f>COUNTIF(E304:G304,"有")+IF(H304&gt;=6,1,0)+IF(I304&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M304" s="11" t="n"/>
+      <c r="N304" s="13">
+        <f>IF(COUNTA(A304:G304)=0,"",IF(L304&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" s="10" t="n"/>
+      <c r="B305" s="11" t="n"/>
+      <c r="C305" s="11" t="n"/>
+      <c r="D305" s="11" t="n"/>
+      <c r="E305" s="11" t="n"/>
+      <c r="F305" s="11" t="n"/>
+      <c r="G305" s="11" t="n"/>
+      <c r="H305" s="11" t="n"/>
+      <c r="I305" s="11" t="n"/>
+      <c r="J305" s="12" t="n"/>
+      <c r="K305" s="12" t="n"/>
+      <c r="L305" s="13">
+        <f>COUNTIF(E305:G305,"有")+IF(H305&gt;=6,1,0)+IF(I305&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M305" s="11" t="n"/>
+      <c r="N305" s="13">
+        <f>IF(COUNTA(A305:G305)=0,"",IF(L305&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" s="10" t="n"/>
+      <c r="B306" s="11" t="n"/>
+      <c r="C306" s="11" t="n"/>
+      <c r="D306" s="11" t="n"/>
+      <c r="E306" s="11" t="n"/>
+      <c r="F306" s="11" t="n"/>
+      <c r="G306" s="11" t="n"/>
+      <c r="H306" s="11" t="n"/>
+      <c r="I306" s="11" t="n"/>
+      <c r="J306" s="12" t="n"/>
+      <c r="K306" s="12" t="n"/>
+      <c r="L306" s="13">
+        <f>COUNTIF(E306:G306,"有")+IF(H306&gt;=6,1,0)+IF(I306&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M306" s="11" t="n"/>
+      <c r="N306" s="13">
+        <f>IF(COUNTA(A306:G306)=0,"",IF(L306&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" s="10" t="n"/>
+      <c r="B307" s="11" t="n"/>
+      <c r="C307" s="11" t="n"/>
+      <c r="D307" s="11" t="n"/>
+      <c r="E307" s="11" t="n"/>
+      <c r="F307" s="11" t="n"/>
+      <c r="G307" s="11" t="n"/>
+      <c r="H307" s="11" t="n"/>
+      <c r="I307" s="11" t="n"/>
+      <c r="J307" s="12" t="n"/>
+      <c r="K307" s="12" t="n"/>
+      <c r="L307" s="13">
+        <f>COUNTIF(E307:G307,"有")+IF(H307&gt;=6,1,0)+IF(I307&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M307" s="11" t="n"/>
+      <c r="N307" s="13">
+        <f>IF(COUNTA(A307:G307)=0,"",IF(L307&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" s="10" t="n"/>
+      <c r="B308" s="11" t="n"/>
+      <c r="C308" s="11" t="n"/>
+      <c r="D308" s="11" t="n"/>
+      <c r="E308" s="11" t="n"/>
+      <c r="F308" s="11" t="n"/>
+      <c r="G308" s="11" t="n"/>
+      <c r="H308" s="11" t="n"/>
+      <c r="I308" s="11" t="n"/>
+      <c r="J308" s="12" t="n"/>
+      <c r="K308" s="12" t="n"/>
+      <c r="L308" s="13">
+        <f>COUNTIF(E308:G308,"有")+IF(H308&gt;=6,1,0)+IF(I308&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M308" s="11" t="n"/>
+      <c r="N308" s="13">
+        <f>IF(COUNTA(A308:G308)=0,"",IF(L308&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" s="10" t="n"/>
+      <c r="B309" s="11" t="n"/>
+      <c r="C309" s="11" t="n"/>
+      <c r="D309" s="11" t="n"/>
+      <c r="E309" s="11" t="n"/>
+      <c r="F309" s="11" t="n"/>
+      <c r="G309" s="11" t="n"/>
+      <c r="H309" s="11" t="n"/>
+      <c r="I309" s="11" t="n"/>
+      <c r="J309" s="12" t="n"/>
+      <c r="K309" s="12" t="n"/>
+      <c r="L309" s="13">
+        <f>COUNTIF(E309:G309,"有")+IF(H309&gt;=6,1,0)+IF(I309&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M309" s="11" t="n"/>
+      <c r="N309" s="13">
+        <f>IF(COUNTA(A309:G309)=0,"",IF(L309&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" s="10" t="n"/>
+      <c r="B310" s="11" t="n"/>
+      <c r="C310" s="11" t="n"/>
+      <c r="D310" s="11" t="n"/>
+      <c r="E310" s="11" t="n"/>
+      <c r="F310" s="11" t="n"/>
+      <c r="G310" s="11" t="n"/>
+      <c r="H310" s="11" t="n"/>
+      <c r="I310" s="11" t="n"/>
+      <c r="J310" s="12" t="n"/>
+      <c r="K310" s="12" t="n"/>
+      <c r="L310" s="13">
+        <f>COUNTIF(E310:G310,"有")+IF(H310&gt;=6,1,0)+IF(I310&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M310" s="11" t="n"/>
+      <c r="N310" s="13">
+        <f>IF(COUNTA(A310:G310)=0,"",IF(L310&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" s="10" t="n"/>
+      <c r="B311" s="11" t="n"/>
+      <c r="C311" s="11" t="n"/>
+      <c r="D311" s="11" t="n"/>
+      <c r="E311" s="11" t="n"/>
+      <c r="F311" s="11" t="n"/>
+      <c r="G311" s="11" t="n"/>
+      <c r="H311" s="11" t="n"/>
+      <c r="I311" s="11" t="n"/>
+      <c r="J311" s="12" t="n"/>
+      <c r="K311" s="12" t="n"/>
+      <c r="L311" s="13">
+        <f>COUNTIF(E311:G311,"有")+IF(H311&gt;=6,1,0)+IF(I311&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M311" s="11" t="n"/>
+      <c r="N311" s="13">
+        <f>IF(COUNTA(A311:G311)=0,"",IF(L311&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" s="10" t="n"/>
+      <c r="B312" s="11" t="n"/>
+      <c r="C312" s="11" t="n"/>
+      <c r="D312" s="11" t="n"/>
+      <c r="E312" s="11" t="n"/>
+      <c r="F312" s="11" t="n"/>
+      <c r="G312" s="11" t="n"/>
+      <c r="H312" s="11" t="n"/>
+      <c r="I312" s="11" t="n"/>
+      <c r="J312" s="12" t="n"/>
+      <c r="K312" s="12" t="n"/>
+      <c r="L312" s="13">
+        <f>COUNTIF(E312:G312,"有")+IF(H312&gt;=6,1,0)+IF(I312&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M312" s="11" t="n"/>
+      <c r="N312" s="13">
+        <f>IF(COUNTA(A312:G312)=0,"",IF(L312&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" s="10" t="n"/>
+      <c r="B313" s="11" t="n"/>
+      <c r="C313" s="11" t="n"/>
+      <c r="D313" s="11" t="n"/>
+      <c r="E313" s="11" t="n"/>
+      <c r="F313" s="11" t="n"/>
+      <c r="G313" s="11" t="n"/>
+      <c r="H313" s="11" t="n"/>
+      <c r="I313" s="11" t="n"/>
+      <c r="J313" s="12" t="n"/>
+      <c r="K313" s="12" t="n"/>
+      <c r="L313" s="13">
+        <f>COUNTIF(E313:G313,"有")+IF(H313&gt;=6,1,0)+IF(I313&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M313" s="11" t="n"/>
+      <c r="N313" s="13">
+        <f>IF(COUNTA(A313:G313)=0,"",IF(L313&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" s="10" t="n"/>
+      <c r="B314" s="11" t="n"/>
+      <c r="C314" s="11" t="n"/>
+      <c r="D314" s="11" t="n"/>
+      <c r="E314" s="11" t="n"/>
+      <c r="F314" s="11" t="n"/>
+      <c r="G314" s="11" t="n"/>
+      <c r="H314" s="11" t="n"/>
+      <c r="I314" s="11" t="n"/>
+      <c r="J314" s="12" t="n"/>
+      <c r="K314" s="12" t="n"/>
+      <c r="L314" s="13">
+        <f>COUNTIF(E314:G314,"有")+IF(H314&gt;=6,1,0)+IF(I314&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M314" s="11" t="n"/>
+      <c r="N314" s="13">
+        <f>IF(COUNTA(A314:G314)=0,"",IF(L314&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" s="10" t="n"/>
+      <c r="B315" s="11" t="n"/>
+      <c r="C315" s="11" t="n"/>
+      <c r="D315" s="11" t="n"/>
+      <c r="E315" s="11" t="n"/>
+      <c r="F315" s="11" t="n"/>
+      <c r="G315" s="11" t="n"/>
+      <c r="H315" s="11" t="n"/>
+      <c r="I315" s="11" t="n"/>
+      <c r="J315" s="12" t="n"/>
+      <c r="K315" s="12" t="n"/>
+      <c r="L315" s="13">
+        <f>COUNTIF(E315:G315,"有")+IF(H315&gt;=6,1,0)+IF(I315&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M315" s="11" t="n"/>
+      <c r="N315" s="13">
+        <f>IF(COUNTA(A315:G315)=0,"",IF(L315&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" s="10" t="n"/>
+      <c r="B316" s="11" t="n"/>
+      <c r="C316" s="11" t="n"/>
+      <c r="D316" s="11" t="n"/>
+      <c r="E316" s="11" t="n"/>
+      <c r="F316" s="11" t="n"/>
+      <c r="G316" s="11" t="n"/>
+      <c r="H316" s="11" t="n"/>
+      <c r="I316" s="11" t="n"/>
+      <c r="J316" s="12" t="n"/>
+      <c r="K316" s="12" t="n"/>
+      <c r="L316" s="13">
+        <f>COUNTIF(E316:G316,"有")+IF(H316&gt;=6,1,0)+IF(I316&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M316" s="11" t="n"/>
+      <c r="N316" s="13">
+        <f>IF(COUNTA(A316:G316)=0,"",IF(L316&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" s="10" t="n"/>
+      <c r="B317" s="11" t="n"/>
+      <c r="C317" s="11" t="n"/>
+      <c r="D317" s="11" t="n"/>
+      <c r="E317" s="11" t="n"/>
+      <c r="F317" s="11" t="n"/>
+      <c r="G317" s="11" t="n"/>
+      <c r="H317" s="11" t="n"/>
+      <c r="I317" s="11" t="n"/>
+      <c r="J317" s="12" t="n"/>
+      <c r="K317" s="12" t="n"/>
+      <c r="L317" s="13">
+        <f>COUNTIF(E317:G317,"有")+IF(H317&gt;=6,1,0)+IF(I317&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M317" s="11" t="n"/>
+      <c r="N317" s="13">
+        <f>IF(COUNTA(A317:G317)=0,"",IF(L317&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" s="10" t="n"/>
+      <c r="B318" s="11" t="n"/>
+      <c r="C318" s="11" t="n"/>
+      <c r="D318" s="11" t="n"/>
+      <c r="E318" s="11" t="n"/>
+      <c r="F318" s="11" t="n"/>
+      <c r="G318" s="11" t="n"/>
+      <c r="H318" s="11" t="n"/>
+      <c r="I318" s="11" t="n"/>
+      <c r="J318" s="12" t="n"/>
+      <c r="K318" s="12" t="n"/>
+      <c r="L318" s="13">
+        <f>COUNTIF(E318:G318,"有")+IF(H318&gt;=6,1,0)+IF(I318&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M318" s="11" t="n"/>
+      <c r="N318" s="13">
+        <f>IF(COUNTA(A318:G318)=0,"",IF(L318&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" s="10" t="n"/>
+      <c r="B319" s="11" t="n"/>
+      <c r="C319" s="11" t="n"/>
+      <c r="D319" s="11" t="n"/>
+      <c r="E319" s="11" t="n"/>
+      <c r="F319" s="11" t="n"/>
+      <c r="G319" s="11" t="n"/>
+      <c r="H319" s="11" t="n"/>
+      <c r="I319" s="11" t="n"/>
+      <c r="J319" s="12" t="n"/>
+      <c r="K319" s="12" t="n"/>
+      <c r="L319" s="13">
+        <f>COUNTIF(E319:G319,"有")+IF(H319&gt;=6,1,0)+IF(I319&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M319" s="11" t="n"/>
+      <c r="N319" s="13">
+        <f>IF(COUNTA(A319:G319)=0,"",IF(L319&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" s="10" t="n"/>
+      <c r="B320" s="11" t="n"/>
+      <c r="C320" s="11" t="n"/>
+      <c r="D320" s="11" t="n"/>
+      <c r="E320" s="11" t="n"/>
+      <c r="F320" s="11" t="n"/>
+      <c r="G320" s="11" t="n"/>
+      <c r="H320" s="11" t="n"/>
+      <c r="I320" s="11" t="n"/>
+      <c r="J320" s="12" t="n"/>
+      <c r="K320" s="12" t="n"/>
+      <c r="L320" s="13">
+        <f>COUNTIF(E320:G320,"有")+IF(H320&gt;=6,1,0)+IF(I320&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M320" s="11" t="n"/>
+      <c r="N320" s="13">
+        <f>IF(COUNTA(A320:G320)=0,"",IF(L320&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" s="10" t="n"/>
+      <c r="B321" s="11" t="n"/>
+      <c r="C321" s="11" t="n"/>
+      <c r="D321" s="11" t="n"/>
+      <c r="E321" s="11" t="n"/>
+      <c r="F321" s="11" t="n"/>
+      <c r="G321" s="11" t="n"/>
+      <c r="H321" s="11" t="n"/>
+      <c r="I321" s="11" t="n"/>
+      <c r="J321" s="12" t="n"/>
+      <c r="K321" s="12" t="n"/>
+      <c r="L321" s="13">
+        <f>COUNTIF(E321:G321,"有")+IF(H321&gt;=6,1,0)+IF(I321&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M321" s="11" t="n"/>
+      <c r="N321" s="13">
+        <f>IF(COUNTA(A321:G321)=0,"",IF(L321&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" s="10" t="n"/>
+      <c r="B322" s="11" t="n"/>
+      <c r="C322" s="11" t="n"/>
+      <c r="D322" s="11" t="n"/>
+      <c r="E322" s="11" t="n"/>
+      <c r="F322" s="11" t="n"/>
+      <c r="G322" s="11" t="n"/>
+      <c r="H322" s="11" t="n"/>
+      <c r="I322" s="11" t="n"/>
+      <c r="J322" s="12" t="n"/>
+      <c r="K322" s="12" t="n"/>
+      <c r="L322" s="13">
+        <f>COUNTIF(E322:G322,"有")+IF(H322&gt;=6,1,0)+IF(I322&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M322" s="11" t="n"/>
+      <c r="N322" s="13">
+        <f>IF(COUNTA(A322:G322)=0,"",IF(L322&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" s="10" t="n"/>
+      <c r="B323" s="11" t="n"/>
+      <c r="C323" s="11" t="n"/>
+      <c r="D323" s="11" t="n"/>
+      <c r="E323" s="11" t="n"/>
+      <c r="F323" s="11" t="n"/>
+      <c r="G323" s="11" t="n"/>
+      <c r="H323" s="11" t="n"/>
+      <c r="I323" s="11" t="n"/>
+      <c r="J323" s="12" t="n"/>
+      <c r="K323" s="12" t="n"/>
+      <c r="L323" s="13">
+        <f>COUNTIF(E323:G323,"有")+IF(H323&gt;=6,1,0)+IF(I323&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M323" s="11" t="n"/>
+      <c r="N323" s="13">
+        <f>IF(COUNTA(A323:G323)=0,"",IF(L323&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" s="10" t="n"/>
+      <c r="B324" s="11" t="n"/>
+      <c r="C324" s="11" t="n"/>
+      <c r="D324" s="11" t="n"/>
+      <c r="E324" s="11" t="n"/>
+      <c r="F324" s="11" t="n"/>
+      <c r="G324" s="11" t="n"/>
+      <c r="H324" s="11" t="n"/>
+      <c r="I324" s="11" t="n"/>
+      <c r="J324" s="12" t="n"/>
+      <c r="K324" s="12" t="n"/>
+      <c r="L324" s="13">
+        <f>COUNTIF(E324:G324,"有")+IF(H324&gt;=6,1,0)+IF(I324&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M324" s="11" t="n"/>
+      <c r="N324" s="13">
+        <f>IF(COUNTA(A324:G324)=0,"",IF(L324&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" s="10" t="n"/>
+      <c r="B325" s="11" t="n"/>
+      <c r="C325" s="11" t="n"/>
+      <c r="D325" s="11" t="n"/>
+      <c r="E325" s="11" t="n"/>
+      <c r="F325" s="11" t="n"/>
+      <c r="G325" s="11" t="n"/>
+      <c r="H325" s="11" t="n"/>
+      <c r="I325" s="11" t="n"/>
+      <c r="J325" s="12" t="n"/>
+      <c r="K325" s="12" t="n"/>
+      <c r="L325" s="13">
+        <f>COUNTIF(E325:G325,"有")+IF(H325&gt;=6,1,0)+IF(I325&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M325" s="11" t="n"/>
+      <c r="N325" s="13">
+        <f>IF(COUNTA(A325:G325)=0,"",IF(L325&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" s="10" t="n"/>
+      <c r="B326" s="11" t="n"/>
+      <c r="C326" s="11" t="n"/>
+      <c r="D326" s="11" t="n"/>
+      <c r="E326" s="11" t="n"/>
+      <c r="F326" s="11" t="n"/>
+      <c r="G326" s="11" t="n"/>
+      <c r="H326" s="11" t="n"/>
+      <c r="I326" s="11" t="n"/>
+      <c r="J326" s="12" t="n"/>
+      <c r="K326" s="12" t="n"/>
+      <c r="L326" s="13">
+        <f>COUNTIF(E326:G326,"有")+IF(H326&gt;=6,1,0)+IF(I326&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M326" s="11" t="n"/>
+      <c r="N326" s="13">
+        <f>IF(COUNTA(A326:G326)=0,"",IF(L326&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" s="10" t="n"/>
+      <c r="B327" s="11" t="n"/>
+      <c r="C327" s="11" t="n"/>
+      <c r="D327" s="11" t="n"/>
+      <c r="E327" s="11" t="n"/>
+      <c r="F327" s="11" t="n"/>
+      <c r="G327" s="11" t="n"/>
+      <c r="H327" s="11" t="n"/>
+      <c r="I327" s="11" t="n"/>
+      <c r="J327" s="12" t="n"/>
+      <c r="K327" s="12" t="n"/>
+      <c r="L327" s="13">
+        <f>COUNTIF(E327:G327,"有")+IF(H327&gt;=6,1,0)+IF(I327&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M327" s="11" t="n"/>
+      <c r="N327" s="13">
+        <f>IF(COUNTA(A327:G327)=0,"",IF(L327&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" s="10" t="n"/>
+      <c r="B328" s="11" t="n"/>
+      <c r="C328" s="11" t="n"/>
+      <c r="D328" s="11" t="n"/>
+      <c r="E328" s="11" t="n"/>
+      <c r="F328" s="11" t="n"/>
+      <c r="G328" s="11" t="n"/>
+      <c r="H328" s="11" t="n"/>
+      <c r="I328" s="11" t="n"/>
+      <c r="J328" s="12" t="n"/>
+      <c r="K328" s="12" t="n"/>
+      <c r="L328" s="13">
+        <f>COUNTIF(E328:G328,"有")+IF(H328&gt;=6,1,0)+IF(I328&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M328" s="11" t="n"/>
+      <c r="N328" s="13">
+        <f>IF(COUNTA(A328:G328)=0,"",IF(L328&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" s="10" t="n"/>
+      <c r="B329" s="11" t="n"/>
+      <c r="C329" s="11" t="n"/>
+      <c r="D329" s="11" t="n"/>
+      <c r="E329" s="11" t="n"/>
+      <c r="F329" s="11" t="n"/>
+      <c r="G329" s="11" t="n"/>
+      <c r="H329" s="11" t="n"/>
+      <c r="I329" s="11" t="n"/>
+      <c r="J329" s="12" t="n"/>
+      <c r="K329" s="12" t="n"/>
+      <c r="L329" s="13">
+        <f>COUNTIF(E329:G329,"有")+IF(H329&gt;=6,1,0)+IF(I329&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M329" s="11" t="n"/>
+      <c r="N329" s="13">
+        <f>IF(COUNTA(A329:G329)=0,"",IF(L329&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" s="10" t="n"/>
+      <c r="B330" s="11" t="n"/>
+      <c r="C330" s="11" t="n"/>
+      <c r="D330" s="11" t="n"/>
+      <c r="E330" s="11" t="n"/>
+      <c r="F330" s="11" t="n"/>
+      <c r="G330" s="11" t="n"/>
+      <c r="H330" s="11" t="n"/>
+      <c r="I330" s="11" t="n"/>
+      <c r="J330" s="12" t="n"/>
+      <c r="K330" s="12" t="n"/>
+      <c r="L330" s="13">
+        <f>COUNTIF(E330:G330,"有")+IF(H330&gt;=6,1,0)+IF(I330&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M330" s="11" t="n"/>
+      <c r="N330" s="13">
+        <f>IF(COUNTA(A330:G330)=0,"",IF(L330&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" s="10" t="n"/>
+      <c r="B331" s="11" t="n"/>
+      <c r="C331" s="11" t="n"/>
+      <c r="D331" s="11" t="n"/>
+      <c r="E331" s="11" t="n"/>
+      <c r="F331" s="11" t="n"/>
+      <c r="G331" s="11" t="n"/>
+      <c r="H331" s="11" t="n"/>
+      <c r="I331" s="11" t="n"/>
+      <c r="J331" s="12" t="n"/>
+      <c r="K331" s="12" t="n"/>
+      <c r="L331" s="13">
+        <f>COUNTIF(E331:G331,"有")+IF(H331&gt;=6,1,0)+IF(I331&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M331" s="11" t="n"/>
+      <c r="N331" s="13">
+        <f>IF(COUNTA(A331:G331)=0,"",IF(L331&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" s="10" t="n"/>
+      <c r="B332" s="11" t="n"/>
+      <c r="C332" s="11" t="n"/>
+      <c r="D332" s="11" t="n"/>
+      <c r="E332" s="11" t="n"/>
+      <c r="F332" s="11" t="n"/>
+      <c r="G332" s="11" t="n"/>
+      <c r="H332" s="11" t="n"/>
+      <c r="I332" s="11" t="n"/>
+      <c r="J332" s="12" t="n"/>
+      <c r="K332" s="12" t="n"/>
+      <c r="L332" s="13">
+        <f>COUNTIF(E332:G332,"有")+IF(H332&gt;=6,1,0)+IF(I332&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M332" s="11" t="n"/>
+      <c r="N332" s="13">
+        <f>IF(COUNTA(A332:G332)=0,"",IF(L332&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" s="10" t="n"/>
+      <c r="B333" s="11" t="n"/>
+      <c r="C333" s="11" t="n"/>
+      <c r="D333" s="11" t="n"/>
+      <c r="E333" s="11" t="n"/>
+      <c r="F333" s="11" t="n"/>
+      <c r="G333" s="11" t="n"/>
+      <c r="H333" s="11" t="n"/>
+      <c r="I333" s="11" t="n"/>
+      <c r="J333" s="12" t="n"/>
+      <c r="K333" s="12" t="n"/>
+      <c r="L333" s="13">
+        <f>COUNTIF(E333:G333,"有")+IF(H333&gt;=6,1,0)+IF(I333&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M333" s="11" t="n"/>
+      <c r="N333" s="13">
+        <f>IF(COUNTA(A333:G333)=0,"",IF(L333&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" s="10" t="n"/>
+      <c r="B334" s="11" t="n"/>
+      <c r="C334" s="11" t="n"/>
+      <c r="D334" s="11" t="n"/>
+      <c r="E334" s="11" t="n"/>
+      <c r="F334" s="11" t="n"/>
+      <c r="G334" s="11" t="n"/>
+      <c r="H334" s="11" t="n"/>
+      <c r="I334" s="11" t="n"/>
+      <c r="J334" s="12" t="n"/>
+      <c r="K334" s="12" t="n"/>
+      <c r="L334" s="13">
+        <f>COUNTIF(E334:G334,"有")+IF(H334&gt;=6,1,0)+IF(I334&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M334" s="11" t="n"/>
+      <c r="N334" s="13">
+        <f>IF(COUNTA(A334:G334)=0,"",IF(L334&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" s="10" t="n"/>
+      <c r="B335" s="11" t="n"/>
+      <c r="C335" s="11" t="n"/>
+      <c r="D335" s="11" t="n"/>
+      <c r="E335" s="11" t="n"/>
+      <c r="F335" s="11" t="n"/>
+      <c r="G335" s="11" t="n"/>
+      <c r="H335" s="11" t="n"/>
+      <c r="I335" s="11" t="n"/>
+      <c r="J335" s="12" t="n"/>
+      <c r="K335" s="12" t="n"/>
+      <c r="L335" s="13">
+        <f>COUNTIF(E335:G335,"有")+IF(H335&gt;=6,1,0)+IF(I335&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M335" s="11" t="n"/>
+      <c r="N335" s="13">
+        <f>IF(COUNTA(A335:G335)=0,"",IF(L335&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" s="10" t="n"/>
+      <c r="B336" s="11" t="n"/>
+      <c r="C336" s="11" t="n"/>
+      <c r="D336" s="11" t="n"/>
+      <c r="E336" s="11" t="n"/>
+      <c r="F336" s="11" t="n"/>
+      <c r="G336" s="11" t="n"/>
+      <c r="H336" s="11" t="n"/>
+      <c r="I336" s="11" t="n"/>
+      <c r="J336" s="12" t="n"/>
+      <c r="K336" s="12" t="n"/>
+      <c r="L336" s="13">
+        <f>COUNTIF(E336:G336,"有")+IF(H336&gt;=6,1,0)+IF(I336&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M336" s="11" t="n"/>
+      <c r="N336" s="13">
+        <f>IF(COUNTA(A336:G336)=0,"",IF(L336&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" s="10" t="n"/>
+      <c r="B337" s="11" t="n"/>
+      <c r="C337" s="11" t="n"/>
+      <c r="D337" s="11" t="n"/>
+      <c r="E337" s="11" t="n"/>
+      <c r="F337" s="11" t="n"/>
+      <c r="G337" s="11" t="n"/>
+      <c r="H337" s="11" t="n"/>
+      <c r="I337" s="11" t="n"/>
+      <c r="J337" s="12" t="n"/>
+      <c r="K337" s="12" t="n"/>
+      <c r="L337" s="13">
+        <f>COUNTIF(E337:G337,"有")+IF(H337&gt;=6,1,0)+IF(I337&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M337" s="11" t="n"/>
+      <c r="N337" s="13">
+        <f>IF(COUNTA(A337:G337)=0,"",IF(L337&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" s="10" t="n"/>
+      <c r="B338" s="11" t="n"/>
+      <c r="C338" s="11" t="n"/>
+      <c r="D338" s="11" t="n"/>
+      <c r="E338" s="11" t="n"/>
+      <c r="F338" s="11" t="n"/>
+      <c r="G338" s="11" t="n"/>
+      <c r="H338" s="11" t="n"/>
+      <c r="I338" s="11" t="n"/>
+      <c r="J338" s="12" t="n"/>
+      <c r="K338" s="12" t="n"/>
+      <c r="L338" s="13">
+        <f>COUNTIF(E338:G338,"有")+IF(H338&gt;=6,1,0)+IF(I338&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M338" s="11" t="n"/>
+      <c r="N338" s="13">
+        <f>IF(COUNTA(A338:G338)=0,"",IF(L338&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" s="10" t="n"/>
+      <c r="B339" s="11" t="n"/>
+      <c r="C339" s="11" t="n"/>
+      <c r="D339" s="11" t="n"/>
+      <c r="E339" s="11" t="n"/>
+      <c r="F339" s="11" t="n"/>
+      <c r="G339" s="11" t="n"/>
+      <c r="H339" s="11" t="n"/>
+      <c r="I339" s="11" t="n"/>
+      <c r="J339" s="12" t="n"/>
+      <c r="K339" s="12" t="n"/>
+      <c r="L339" s="13">
+        <f>COUNTIF(E339:G339,"有")+IF(H339&gt;=6,1,0)+IF(I339&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M339" s="11" t="n"/>
+      <c r="N339" s="13">
+        <f>IF(COUNTA(A339:G339)=0,"",IF(L339&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" s="10" t="n"/>
+      <c r="B340" s="11" t="n"/>
+      <c r="C340" s="11" t="n"/>
+      <c r="D340" s="11" t="n"/>
+      <c r="E340" s="11" t="n"/>
+      <c r="F340" s="11" t="n"/>
+      <c r="G340" s="11" t="n"/>
+      <c r="H340" s="11" t="n"/>
+      <c r="I340" s="11" t="n"/>
+      <c r="J340" s="12" t="n"/>
+      <c r="K340" s="12" t="n"/>
+      <c r="L340" s="13">
+        <f>COUNTIF(E340:G340,"有")+IF(H340&gt;=6,1,0)+IF(I340&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M340" s="11" t="n"/>
+      <c r="N340" s="13">
+        <f>IF(COUNTA(A340:G340)=0,"",IF(L340&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" s="10" t="n"/>
+      <c r="B341" s="11" t="n"/>
+      <c r="C341" s="11" t="n"/>
+      <c r="D341" s="11" t="n"/>
+      <c r="E341" s="11" t="n"/>
+      <c r="F341" s="11" t="n"/>
+      <c r="G341" s="11" t="n"/>
+      <c r="H341" s="11" t="n"/>
+      <c r="I341" s="11" t="n"/>
+      <c r="J341" s="12" t="n"/>
+      <c r="K341" s="12" t="n"/>
+      <c r="L341" s="13">
+        <f>COUNTIF(E341:G341,"有")+IF(H341&gt;=6,1,0)+IF(I341&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M341" s="11" t="n"/>
+      <c r="N341" s="13">
+        <f>IF(COUNTA(A341:G341)=0,"",IF(L341&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" s="10" t="n"/>
+      <c r="B342" s="11" t="n"/>
+      <c r="C342" s="11" t="n"/>
+      <c r="D342" s="11" t="n"/>
+      <c r="E342" s="11" t="n"/>
+      <c r="F342" s="11" t="n"/>
+      <c r="G342" s="11" t="n"/>
+      <c r="H342" s="11" t="n"/>
+      <c r="I342" s="11" t="n"/>
+      <c r="J342" s="12" t="n"/>
+      <c r="K342" s="12" t="n"/>
+      <c r="L342" s="13">
+        <f>COUNTIF(E342:G342,"有")+IF(H342&gt;=6,1,0)+IF(I342&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M342" s="11" t="n"/>
+      <c r="N342" s="13">
+        <f>IF(COUNTA(A342:G342)=0,"",IF(L342&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" s="10" t="n"/>
+      <c r="B343" s="11" t="n"/>
+      <c r="C343" s="11" t="n"/>
+      <c r="D343" s="11" t="n"/>
+      <c r="E343" s="11" t="n"/>
+      <c r="F343" s="11" t="n"/>
+      <c r="G343" s="11" t="n"/>
+      <c r="H343" s="11" t="n"/>
+      <c r="I343" s="11" t="n"/>
+      <c r="J343" s="12" t="n"/>
+      <c r="K343" s="12" t="n"/>
+      <c r="L343" s="13">
+        <f>COUNTIF(E343:G343,"有")+IF(H343&gt;=6,1,0)+IF(I343&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M343" s="11" t="n"/>
+      <c r="N343" s="13">
+        <f>IF(COUNTA(A343:G343)=0,"",IF(L343&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" s="10" t="n"/>
+      <c r="B344" s="11" t="n"/>
+      <c r="C344" s="11" t="n"/>
+      <c r="D344" s="11" t="n"/>
+      <c r="E344" s="11" t="n"/>
+      <c r="F344" s="11" t="n"/>
+      <c r="G344" s="11" t="n"/>
+      <c r="H344" s="11" t="n"/>
+      <c r="I344" s="11" t="n"/>
+      <c r="J344" s="12" t="n"/>
+      <c r="K344" s="12" t="n"/>
+      <c r="L344" s="13">
+        <f>COUNTIF(E344:G344,"有")+IF(H344&gt;=6,1,0)+IF(I344&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M344" s="11" t="n"/>
+      <c r="N344" s="13">
+        <f>IF(COUNTA(A344:G344)=0,"",IF(L344&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" s="10" t="n"/>
+      <c r="B345" s="11" t="n"/>
+      <c r="C345" s="11" t="n"/>
+      <c r="D345" s="11" t="n"/>
+      <c r="E345" s="11" t="n"/>
+      <c r="F345" s="11" t="n"/>
+      <c r="G345" s="11" t="n"/>
+      <c r="H345" s="11" t="n"/>
+      <c r="I345" s="11" t="n"/>
+      <c r="J345" s="12" t="n"/>
+      <c r="K345" s="12" t="n"/>
+      <c r="L345" s="13">
+        <f>COUNTIF(E345:G345,"有")+IF(H345&gt;=6,1,0)+IF(I345&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M345" s="11" t="n"/>
+      <c r="N345" s="13">
+        <f>IF(COUNTA(A345:G345)=0,"",IF(L345&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" s="10" t="n"/>
+      <c r="B346" s="11" t="n"/>
+      <c r="C346" s="11" t="n"/>
+      <c r="D346" s="11" t="n"/>
+      <c r="E346" s="11" t="n"/>
+      <c r="F346" s="11" t="n"/>
+      <c r="G346" s="11" t="n"/>
+      <c r="H346" s="11" t="n"/>
+      <c r="I346" s="11" t="n"/>
+      <c r="J346" s="12" t="n"/>
+      <c r="K346" s="12" t="n"/>
+      <c r="L346" s="13">
+        <f>COUNTIF(E346:G346,"有")+IF(H346&gt;=6,1,0)+IF(I346&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M346" s="11" t="n"/>
+      <c r="N346" s="13">
+        <f>IF(COUNTA(A346:G346)=0,"",IF(L346&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" s="10" t="n"/>
+      <c r="B347" s="11" t="n"/>
+      <c r="C347" s="11" t="n"/>
+      <c r="D347" s="11" t="n"/>
+      <c r="E347" s="11" t="n"/>
+      <c r="F347" s="11" t="n"/>
+      <c r="G347" s="11" t="n"/>
+      <c r="H347" s="11" t="n"/>
+      <c r="I347" s="11" t="n"/>
+      <c r="J347" s="12" t="n"/>
+      <c r="K347" s="12" t="n"/>
+      <c r="L347" s="13">
+        <f>COUNTIF(E347:G347,"有")+IF(H347&gt;=6,1,0)+IF(I347&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M347" s="11" t="n"/>
+      <c r="N347" s="13">
+        <f>IF(COUNTA(A347:G347)=0,"",IF(L347&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" s="10" t="n"/>
+      <c r="B348" s="11" t="n"/>
+      <c r="C348" s="11" t="n"/>
+      <c r="D348" s="11" t="n"/>
+      <c r="E348" s="11" t="n"/>
+      <c r="F348" s="11" t="n"/>
+      <c r="G348" s="11" t="n"/>
+      <c r="H348" s="11" t="n"/>
+      <c r="I348" s="11" t="n"/>
+      <c r="J348" s="12" t="n"/>
+      <c r="K348" s="12" t="n"/>
+      <c r="L348" s="13">
+        <f>COUNTIF(E348:G348,"有")+IF(H348&gt;=6,1,0)+IF(I348&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M348" s="11" t="n"/>
+      <c r="N348" s="13">
+        <f>IF(COUNTA(A348:G348)=0,"",IF(L348&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" s="10" t="n"/>
+      <c r="B349" s="11" t="n"/>
+      <c r="C349" s="11" t="n"/>
+      <c r="D349" s="11" t="n"/>
+      <c r="E349" s="11" t="n"/>
+      <c r="F349" s="11" t="n"/>
+      <c r="G349" s="11" t="n"/>
+      <c r="H349" s="11" t="n"/>
+      <c r="I349" s="11" t="n"/>
+      <c r="J349" s="12" t="n"/>
+      <c r="K349" s="12" t="n"/>
+      <c r="L349" s="13">
+        <f>COUNTIF(E349:G349,"有")+IF(H349&gt;=6,1,0)+IF(I349&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M349" s="11" t="n"/>
+      <c r="N349" s="13">
+        <f>IF(COUNTA(A349:G349)=0,"",IF(L349&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" s="10" t="n"/>
+      <c r="B350" s="11" t="n"/>
+      <c r="C350" s="11" t="n"/>
+      <c r="D350" s="11" t="n"/>
+      <c r="E350" s="11" t="n"/>
+      <c r="F350" s="11" t="n"/>
+      <c r="G350" s="11" t="n"/>
+      <c r="H350" s="11" t="n"/>
+      <c r="I350" s="11" t="n"/>
+      <c r="J350" s="12" t="n"/>
+      <c r="K350" s="12" t="n"/>
+      <c r="L350" s="13">
+        <f>COUNTIF(E350:G350,"有")+IF(H350&gt;=6,1,0)+IF(I350&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M350" s="11" t="n"/>
+      <c r="N350" s="13">
+        <f>IF(COUNTA(A350:G350)=0,"",IF(L350&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" s="10" t="n"/>
+      <c r="B351" s="11" t="n"/>
+      <c r="C351" s="11" t="n"/>
+      <c r="D351" s="11" t="n"/>
+      <c r="E351" s="11" t="n"/>
+      <c r="F351" s="11" t="n"/>
+      <c r="G351" s="11" t="n"/>
+      <c r="H351" s="11" t="n"/>
+      <c r="I351" s="11" t="n"/>
+      <c r="J351" s="12" t="n"/>
+      <c r="K351" s="12" t="n"/>
+      <c r="L351" s="13">
+        <f>COUNTIF(E351:G351,"有")+IF(H351&gt;=6,1,0)+IF(I351&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M351" s="11" t="n"/>
+      <c r="N351" s="13">
+        <f>IF(COUNTA(A351:G351)=0,"",IF(L351&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" s="10" t="n"/>
+      <c r="B352" s="11" t="n"/>
+      <c r="C352" s="11" t="n"/>
+      <c r="D352" s="11" t="n"/>
+      <c r="E352" s="11" t="n"/>
+      <c r="F352" s="11" t="n"/>
+      <c r="G352" s="11" t="n"/>
+      <c r="H352" s="11" t="n"/>
+      <c r="I352" s="11" t="n"/>
+      <c r="J352" s="12" t="n"/>
+      <c r="K352" s="12" t="n"/>
+      <c r="L352" s="13">
+        <f>COUNTIF(E352:G352,"有")+IF(H352&gt;=6,1,0)+IF(I352&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M352" s="11" t="n"/>
+      <c r="N352" s="13">
+        <f>IF(COUNTA(A352:G352)=0,"",IF(L352&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" s="10" t="n"/>
+      <c r="B353" s="11" t="n"/>
+      <c r="C353" s="11" t="n"/>
+      <c r="D353" s="11" t="n"/>
+      <c r="E353" s="11" t="n"/>
+      <c r="F353" s="11" t="n"/>
+      <c r="G353" s="11" t="n"/>
+      <c r="H353" s="11" t="n"/>
+      <c r="I353" s="11" t="n"/>
+      <c r="J353" s="12" t="n"/>
+      <c r="K353" s="12" t="n"/>
+      <c r="L353" s="13">
+        <f>COUNTIF(E353:G353,"有")+IF(H353&gt;=6,1,0)+IF(I353&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M353" s="11" t="n"/>
+      <c r="N353" s="13">
+        <f>IF(COUNTA(A353:G353)=0,"",IF(L353&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" s="10" t="n"/>
+      <c r="B354" s="11" t="n"/>
+      <c r="C354" s="11" t="n"/>
+      <c r="D354" s="11" t="n"/>
+      <c r="E354" s="11" t="n"/>
+      <c r="F354" s="11" t="n"/>
+      <c r="G354" s="11" t="n"/>
+      <c r="H354" s="11" t="n"/>
+      <c r="I354" s="11" t="n"/>
+      <c r="J354" s="12" t="n"/>
+      <c r="K354" s="12" t="n"/>
+      <c r="L354" s="13">
+        <f>COUNTIF(E354:G354,"有")+IF(H354&gt;=6,1,0)+IF(I354&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M354" s="11" t="n"/>
+      <c r="N354" s="13">
+        <f>IF(COUNTA(A354:G354)=0,"",IF(L354&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" s="10" t="n"/>
+      <c r="B355" s="11" t="n"/>
+      <c r="C355" s="11" t="n"/>
+      <c r="D355" s="11" t="n"/>
+      <c r="E355" s="11" t="n"/>
+      <c r="F355" s="11" t="n"/>
+      <c r="G355" s="11" t="n"/>
+      <c r="H355" s="11" t="n"/>
+      <c r="I355" s="11" t="n"/>
+      <c r="J355" s="12" t="n"/>
+      <c r="K355" s="12" t="n"/>
+      <c r="L355" s="13">
+        <f>COUNTIF(E355:G355,"有")+IF(H355&gt;=6,1,0)+IF(I355&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M355" s="11" t="n"/>
+      <c r="N355" s="13">
+        <f>IF(COUNTA(A355:G355)=0,"",IF(L355&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" s="10" t="n"/>
+      <c r="B356" s="11" t="n"/>
+      <c r="C356" s="11" t="n"/>
+      <c r="D356" s="11" t="n"/>
+      <c r="E356" s="11" t="n"/>
+      <c r="F356" s="11" t="n"/>
+      <c r="G356" s="11" t="n"/>
+      <c r="H356" s="11" t="n"/>
+      <c r="I356" s="11" t="n"/>
+      <c r="J356" s="12" t="n"/>
+      <c r="K356" s="12" t="n"/>
+      <c r="L356" s="13">
+        <f>COUNTIF(E356:G356,"有")+IF(H356&gt;=6,1,0)+IF(I356&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M356" s="11" t="n"/>
+      <c r="N356" s="13">
+        <f>IF(COUNTA(A356:G356)=0,"",IF(L356&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" s="10" t="n"/>
+      <c r="B357" s="11" t="n"/>
+      <c r="C357" s="11" t="n"/>
+      <c r="D357" s="11" t="n"/>
+      <c r="E357" s="11" t="n"/>
+      <c r="F357" s="11" t="n"/>
+      <c r="G357" s="11" t="n"/>
+      <c r="H357" s="11" t="n"/>
+      <c r="I357" s="11" t="n"/>
+      <c r="J357" s="12" t="n"/>
+      <c r="K357" s="12" t="n"/>
+      <c r="L357" s="13">
+        <f>COUNTIF(E357:G357,"有")+IF(H357&gt;=6,1,0)+IF(I357&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M357" s="11" t="n"/>
+      <c r="N357" s="13">
+        <f>IF(COUNTA(A357:G357)=0,"",IF(L357&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" s="10" t="n"/>
+      <c r="B358" s="11" t="n"/>
+      <c r="C358" s="11" t="n"/>
+      <c r="D358" s="11" t="n"/>
+      <c r="E358" s="11" t="n"/>
+      <c r="F358" s="11" t="n"/>
+      <c r="G358" s="11" t="n"/>
+      <c r="H358" s="11" t="n"/>
+      <c r="I358" s="11" t="n"/>
+      <c r="J358" s="12" t="n"/>
+      <c r="K358" s="12" t="n"/>
+      <c r="L358" s="13">
+        <f>COUNTIF(E358:G358,"有")+IF(H358&gt;=6,1,0)+IF(I358&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M358" s="11" t="n"/>
+      <c r="N358" s="13">
+        <f>IF(COUNTA(A358:G358)=0,"",IF(L358&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" s="10" t="n"/>
+      <c r="B359" s="11" t="n"/>
+      <c r="C359" s="11" t="n"/>
+      <c r="D359" s="11" t="n"/>
+      <c r="E359" s="11" t="n"/>
+      <c r="F359" s="11" t="n"/>
+      <c r="G359" s="11" t="n"/>
+      <c r="H359" s="11" t="n"/>
+      <c r="I359" s="11" t="n"/>
+      <c r="J359" s="12" t="n"/>
+      <c r="K359" s="12" t="n"/>
+      <c r="L359" s="13">
+        <f>COUNTIF(E359:G359,"有")+IF(H359&gt;=6,1,0)+IF(I359&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M359" s="11" t="n"/>
+      <c r="N359" s="13">
+        <f>IF(COUNTA(A359:G359)=0,"",IF(L359&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" s="10" t="n"/>
+      <c r="B360" s="11" t="n"/>
+      <c r="C360" s="11" t="n"/>
+      <c r="D360" s="11" t="n"/>
+      <c r="E360" s="11" t="n"/>
+      <c r="F360" s="11" t="n"/>
+      <c r="G360" s="11" t="n"/>
+      <c r="H360" s="11" t="n"/>
+      <c r="I360" s="11" t="n"/>
+      <c r="J360" s="12" t="n"/>
+      <c r="K360" s="12" t="n"/>
+      <c r="L360" s="13">
+        <f>COUNTIF(E360:G360,"有")+IF(H360&gt;=6,1,0)+IF(I360&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M360" s="11" t="n"/>
+      <c r="N360" s="13">
+        <f>IF(COUNTA(A360:G360)=0,"",IF(L360&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" s="10" t="n"/>
+      <c r="B361" s="11" t="n"/>
+      <c r="C361" s="11" t="n"/>
+      <c r="D361" s="11" t="n"/>
+      <c r="E361" s="11" t="n"/>
+      <c r="F361" s="11" t="n"/>
+      <c r="G361" s="11" t="n"/>
+      <c r="H361" s="11" t="n"/>
+      <c r="I361" s="11" t="n"/>
+      <c r="J361" s="12" t="n"/>
+      <c r="K361" s="12" t="n"/>
+      <c r="L361" s="13">
+        <f>COUNTIF(E361:G361,"有")+IF(H361&gt;=6,1,0)+IF(I361&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M361" s="11" t="n"/>
+      <c r="N361" s="13">
+        <f>IF(COUNTA(A361:G361)=0,"",IF(L361&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" s="10" t="n"/>
+      <c r="B362" s="11" t="n"/>
+      <c r="C362" s="11" t="n"/>
+      <c r="D362" s="11" t="n"/>
+      <c r="E362" s="11" t="n"/>
+      <c r="F362" s="11" t="n"/>
+      <c r="G362" s="11" t="n"/>
+      <c r="H362" s="11" t="n"/>
+      <c r="I362" s="11" t="n"/>
+      <c r="J362" s="12" t="n"/>
+      <c r="K362" s="12" t="n"/>
+      <c r="L362" s="13">
+        <f>COUNTIF(E362:G362,"有")+IF(H362&gt;=6,1,0)+IF(I362&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M362" s="11" t="n"/>
+      <c r="N362" s="13">
+        <f>IF(COUNTA(A362:G362)=0,"",IF(L362&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" s="10" t="n"/>
+      <c r="B363" s="11" t="n"/>
+      <c r="C363" s="11" t="n"/>
+      <c r="D363" s="11" t="n"/>
+      <c r="E363" s="11" t="n"/>
+      <c r="F363" s="11" t="n"/>
+      <c r="G363" s="11" t="n"/>
+      <c r="H363" s="11" t="n"/>
+      <c r="I363" s="11" t="n"/>
+      <c r="J363" s="12" t="n"/>
+      <c r="K363" s="12" t="n"/>
+      <c r="L363" s="13">
+        <f>COUNTIF(E363:G363,"有")+IF(H363&gt;=6,1,0)+IF(I363&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M363" s="11" t="n"/>
+      <c r="N363" s="13">
+        <f>IF(COUNTA(A363:G363)=0,"",IF(L363&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" s="10" t="n"/>
+      <c r="B364" s="11" t="n"/>
+      <c r="C364" s="11" t="n"/>
+      <c r="D364" s="11" t="n"/>
+      <c r="E364" s="11" t="n"/>
+      <c r="F364" s="11" t="n"/>
+      <c r="G364" s="11" t="n"/>
+      <c r="H364" s="11" t="n"/>
+      <c r="I364" s="11" t="n"/>
+      <c r="J364" s="12" t="n"/>
+      <c r="K364" s="12" t="n"/>
+      <c r="L364" s="13">
+        <f>COUNTIF(E364:G364,"有")+IF(H364&gt;=6,1,0)+IF(I364&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M364" s="11" t="n"/>
+      <c r="N364" s="13">
+        <f>IF(COUNTA(A364:G364)=0,"",IF(L364&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" s="10" t="n"/>
+      <c r="B365" s="11" t="n"/>
+      <c r="C365" s="11" t="n"/>
+      <c r="D365" s="11" t="n"/>
+      <c r="E365" s="11" t="n"/>
+      <c r="F365" s="11" t="n"/>
+      <c r="G365" s="11" t="n"/>
+      <c r="H365" s="11" t="n"/>
+      <c r="I365" s="11" t="n"/>
+      <c r="J365" s="12" t="n"/>
+      <c r="K365" s="12" t="n"/>
+      <c r="L365" s="13">
+        <f>COUNTIF(E365:G365,"有")+IF(H365&gt;=6,1,0)+IF(I365&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M365" s="11" t="n"/>
+      <c r="N365" s="13">
+        <f>IF(COUNTA(A365:G365)=0,"",IF(L365&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" s="10" t="n"/>
+      <c r="B366" s="11" t="n"/>
+      <c r="C366" s="11" t="n"/>
+      <c r="D366" s="11" t="n"/>
+      <c r="E366" s="11" t="n"/>
+      <c r="F366" s="11" t="n"/>
+      <c r="G366" s="11" t="n"/>
+      <c r="H366" s="11" t="n"/>
+      <c r="I366" s="11" t="n"/>
+      <c r="J366" s="12" t="n"/>
+      <c r="K366" s="12" t="n"/>
+      <c r="L366" s="13">
+        <f>COUNTIF(E366:G366,"有")+IF(H366&gt;=6,1,0)+IF(I366&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M366" s="11" t="n"/>
+      <c r="N366" s="13">
+        <f>IF(COUNTA(A366:G366)=0,"",IF(L366&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" s="10" t="n"/>
+      <c r="B367" s="11" t="n"/>
+      <c r="C367" s="11" t="n"/>
+      <c r="D367" s="11" t="n"/>
+      <c r="E367" s="11" t="n"/>
+      <c r="F367" s="11" t="n"/>
+      <c r="G367" s="11" t="n"/>
+      <c r="H367" s="11" t="n"/>
+      <c r="I367" s="11" t="n"/>
+      <c r="J367" s="12" t="n"/>
+      <c r="K367" s="12" t="n"/>
+      <c r="L367" s="13">
+        <f>COUNTIF(E367:G367,"有")+IF(H367&gt;=6,1,0)+IF(I367&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M367" s="11" t="n"/>
+      <c r="N367" s="13">
+        <f>IF(COUNTA(A367:G367)=0,"",IF(L367&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" s="10" t="n"/>
+      <c r="B368" s="11" t="n"/>
+      <c r="C368" s="11" t="n"/>
+      <c r="D368" s="11" t="n"/>
+      <c r="E368" s="11" t="n"/>
+      <c r="F368" s="11" t="n"/>
+      <c r="G368" s="11" t="n"/>
+      <c r="H368" s="11" t="n"/>
+      <c r="I368" s="11" t="n"/>
+      <c r="J368" s="12" t="n"/>
+      <c r="K368" s="12" t="n"/>
+      <c r="L368" s="13">
+        <f>COUNTIF(E368:G368,"有")+IF(H368&gt;=6,1,0)+IF(I368&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M368" s="11" t="n"/>
+      <c r="N368" s="13">
+        <f>IF(COUNTA(A368:G368)=0,"",IF(L368&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" s="10" t="n"/>
+      <c r="B369" s="11" t="n"/>
+      <c r="C369" s="11" t="n"/>
+      <c r="D369" s="11" t="n"/>
+      <c r="E369" s="11" t="n"/>
+      <c r="F369" s="11" t="n"/>
+      <c r="G369" s="11" t="n"/>
+      <c r="H369" s="11" t="n"/>
+      <c r="I369" s="11" t="n"/>
+      <c r="J369" s="12" t="n"/>
+      <c r="K369" s="12" t="n"/>
+      <c r="L369" s="13">
+        <f>COUNTIF(E369:G369,"有")+IF(H369&gt;=6,1,0)+IF(I369&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="M369" s="11" t="n"/>
+      <c r="N369" s="13">
+        <f>IF(COUNTA(A369:G369)=0,"",IF(L369&gt;=2,"完成","再觀察"))</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:N204"/>
+  <autoFilter ref="A4:N369"/>
   <mergeCells count="2">
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="A1:N1"/>

</xml_diff>